<commit_message>
OEMiROT (NTZ): Add KEIL project for OEMiROT Loader and fine tune App
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H563ZI/Applications/ROT_NTZ/OEMiROT_NTZ_flash_layout.xlsx
+++ b/Projects/NUCLEO-H563ZI/Applications/ROT_NTZ/OEMiROT_NTZ_flash_layout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ST\Cube\Cube1\STM32CubeH5\Projects\NUCLEO-H563ZI\Applications\ROT_NTZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D11B675-5CB4-4D8D-BB9A-8B04B1C110FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24400E7-1C51-415F-BDD4-B7C8C0861598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{973ADE99-8809-4282-875C-44A8EA15E93C}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="80">
   <si>
     <t>offset</t>
   </si>
@@ -295,6 +295,15 @@
   </si>
   <si>
     <t>UART Ymodem loader as example</t>
+  </si>
+  <si>
+    <t>Must be multiple of page size (2000)</t>
+  </si>
+  <si>
+    <t>App Active (Max)</t>
+  </si>
+  <si>
+    <t>App Download (Max)</t>
   </si>
 </sst>
 </file>
@@ -331,12 +340,24 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -403,7 +424,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -485,11 +506,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -877,7 +924,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5EEE003-AB81-416D-8FF7-83C8B34AB91C}">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -980,6 +1027,9 @@
         <f>IF(($B$10="Y"),$B$5,0)</f>
         <v>2000</v>
       </c>
+      <c r="C11" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>
@@ -1038,7 +1088,7 @@
         <f>DEC2HEX(HEX2DEC(D14)+HEX2DEC(F14)-1)</f>
         <v>8017FFF</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="10">
         <v>18000</v>
       </c>
       <c r="G14" s="3">
@@ -1149,7 +1199,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="B17" s="3">
         <v>0</v>
@@ -1166,7 +1216,7 @@
         <f t="shared" si="0"/>
         <v>810FFFF</v>
       </c>
-      <c r="F17" s="3" t="str">
+      <c r="F17" s="31" t="str">
         <f>DEC2HEX(IF($B$6="N",ROUNDDOWN((HEX2DEC(B4)-HEX2DEC(F14)-HEX2DEC(F15)-HEX2DEC(F20)-HEX2DEC(F16)-HEX2DEC(F19))/2/HEX2DEC($B$5),0)*HEX2DEC($B$5),(HEX2DEC(B4)-HEX2DEC(F14)-HEX2DEC(F15)-HEX2DEC(F20)-HEX2DEC(F16)-HEX2DEC(F19))))</f>
         <v>E6000</v>
       </c>
@@ -1192,7 +1242,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>13</v>
+        <v>79</v>
       </c>
       <c r="B18" s="3">
         <v>2</v>
@@ -1209,7 +1259,7 @@
         <f t="shared" si="0"/>
         <v>81F5FFF</v>
       </c>
-      <c r="F18" s="3" t="str">
+      <c r="F18" s="31" t="str">
         <f>IF($B$6="N",F17,0)</f>
         <v>E6000</v>
       </c>
@@ -1295,7 +1345,7 @@
         <f t="shared" si="0"/>
         <v>81FFFFF</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="10">
         <f>$B$9</f>
         <v>8000</v>
       </c>
@@ -1352,7 +1402,7 @@
         <v>21</v>
       </c>
       <c r="F22" s="13">
-        <f>B4</f>
+        <f>$B$4</f>
         <v>200000</v>
       </c>
       <c r="G22" s="4">
@@ -1389,16 +1439,420 @@
         <v>0</v>
       </c>
     </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="J26" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="K26" s="26" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C27" s="3">
+        <v>0</v>
+      </c>
+      <c r="D27" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C27))</f>
+        <v>8000000</v>
+      </c>
+      <c r="E27" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC(D27)+HEX2DEC(F27)-1)</f>
+        <v>8017FFF</v>
+      </c>
+      <c r="F27" s="10">
+        <v>18000</v>
+      </c>
+      <c r="G27" s="3">
+        <f>H27/1024</f>
+        <v>96</v>
+      </c>
+      <c r="H27" s="2">
+        <f>HEX2DEC(F27)</f>
+        <v>98304</v>
+      </c>
+      <c r="I27" s="17">
+        <f>H27/HEX2DEC($B$5)</f>
+        <v>12</v>
+      </c>
+      <c r="J27" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC(C27)+HEX2DEC(F27))</f>
+        <v>18000</v>
+      </c>
+      <c r="D28" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C28))</f>
+        <v>8018000</v>
+      </c>
+      <c r="E28" s="3" t="str">
+        <f t="shared" ref="E28:E33" si="7">DEC2HEX(HEX2DEC(D28)+HEX2DEC(F28)-1)</f>
+        <v>8027FFF</v>
+      </c>
+      <c r="F28" s="3">
+        <f>IF(($B$6="N"),IF($B$7="N",10000,0),0)</f>
+        <v>10000</v>
+      </c>
+      <c r="G28" s="3">
+        <f t="shared" ref="G28:G36" si="8">H28/1024</f>
+        <v>64</v>
+      </c>
+      <c r="H28" s="2">
+        <f t="shared" ref="H28:H32" si="9">HEX2DEC(F28)</f>
+        <v>65536</v>
+      </c>
+      <c r="I28" s="17">
+        <f t="shared" ref="I28:I32" si="10">H28/HEX2DEC($B$5)</f>
+        <v>8</v>
+      </c>
+      <c r="J28" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="K28" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A29" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" s="3">
+        <v>4</v>
+      </c>
+      <c r="C29" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC(C28)+HEX2DEC(F28))</f>
+        <v>28000</v>
+      </c>
+      <c r="D29" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C29))</f>
+        <v>8028000</v>
+      </c>
+      <c r="E29" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>8029FFF</v>
+      </c>
+      <c r="F29" s="3">
+        <f>$B$11</f>
+        <v>2000</v>
+      </c>
+      <c r="G29" s="3">
+        <f t="shared" si="8"/>
+        <v>8</v>
+      </c>
+      <c r="H29" s="2">
+        <f t="shared" si="9"/>
+        <v>8192</v>
+      </c>
+      <c r="I29" s="17">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="J29" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="K29" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" s="3">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="str">
+        <f t="shared" ref="C30:C32" si="11">DEC2HEX(HEX2DEC(C29)+HEX2DEC(F29))</f>
+        <v>2A000</v>
+      </c>
+      <c r="D30" s="3" t="str">
+        <f t="shared" ref="D30:D32" si="12">DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C30))</f>
+        <v>802A000</v>
+      </c>
+      <c r="E30" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>803FFFF</v>
+      </c>
+      <c r="F30" s="32">
+        <v>16000</v>
+      </c>
+      <c r="G30" s="3">
+        <f t="shared" si="8"/>
+        <v>88</v>
+      </c>
+      <c r="H30" s="2">
+        <f t="shared" si="9"/>
+        <v>90112</v>
+      </c>
+      <c r="I30" s="17">
+        <f t="shared" si="10"/>
+        <v>11</v>
+      </c>
+      <c r="J30" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="K30" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" s="3">
+        <v>2</v>
+      </c>
+      <c r="C31" s="3" t="str">
+        <f t="shared" si="11"/>
+        <v>40000</v>
+      </c>
+      <c r="D31" s="3" t="str">
+        <f t="shared" si="12"/>
+        <v>8040000</v>
+      </c>
+      <c r="E31" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>8055FFF</v>
+      </c>
+      <c r="F31" s="32">
+        <f>IF($B$6="N",F30,0)</f>
+        <v>16000</v>
+      </c>
+      <c r="G31" s="3">
+        <f t="shared" si="8"/>
+        <v>88</v>
+      </c>
+      <c r="H31" s="2">
+        <f t="shared" si="9"/>
+        <v>90112</v>
+      </c>
+      <c r="I31" s="17">
+        <f t="shared" si="10"/>
+        <v>11</v>
+      </c>
+      <c r="J31" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="K31" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B32" s="3">
+        <v>6</v>
+      </c>
+      <c r="C32" s="3" t="str">
+        <f t="shared" si="11"/>
+        <v>56000</v>
+      </c>
+      <c r="D32" s="3" t="str">
+        <f t="shared" si="12"/>
+        <v>8056000</v>
+      </c>
+      <c r="E32" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>8057FFF</v>
+      </c>
+      <c r="F32" s="3">
+        <f>IF($B$10="Y",F29,0)</f>
+        <v>2000</v>
+      </c>
+      <c r="G32" s="3">
+        <f t="shared" si="8"/>
+        <v>8</v>
+      </c>
+      <c r="H32" s="2">
+        <f t="shared" si="9"/>
+        <v>8192</v>
+      </c>
+      <c r="I32" s="17">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="J32" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="K32" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC(C32)+HEX2DEC(F32))</f>
+        <v>58000</v>
+      </c>
+      <c r="D33" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C33))</f>
+        <v>8058000</v>
+      </c>
+      <c r="E33" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>805FFFF</v>
+      </c>
+      <c r="F33" s="10">
+        <f>$B$9</f>
+        <v>8000</v>
+      </c>
+      <c r="G33" s="3">
+        <f>H33/1024</f>
+        <v>32</v>
+      </c>
+      <c r="H33" s="2">
+        <f>HEX2DEC(F33)</f>
+        <v>32768</v>
+      </c>
+      <c r="I33" s="17">
+        <f>H33/HEX2DEC($B$5)</f>
+        <v>4</v>
+      </c>
+      <c r="J33" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="K33" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="12" t="str">
+        <f>DEC2HEX(H34)</f>
+        <v>60000</v>
+      </c>
+      <c r="G34" s="4">
+        <f t="shared" si="8"/>
+        <v>384</v>
+      </c>
+      <c r="H34" s="13">
+        <f>SUM(H27:H33)</f>
+        <v>393216</v>
+      </c>
+      <c r="I34">
+        <f>H34/HEX2DEC($B$5)</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B35" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="13">
+        <f>$B$4</f>
+        <v>200000</v>
+      </c>
+      <c r="G35" s="4">
+        <f t="shared" si="8"/>
+        <v>2048</v>
+      </c>
+      <c r="H35" s="13">
+        <f>HEX2DEC(F35)</f>
+        <v>2097152</v>
+      </c>
+      <c r="I35">
+        <f t="shared" ref="I35:I36" si="13">H35/HEX2DEC($B$5)</f>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F36" s="13" t="str">
+        <f>DEC2HEX(H36)</f>
+        <v>1A0000</v>
+      </c>
+      <c r="G36" s="4">
+        <f t="shared" si="8"/>
+        <v>1664</v>
+      </c>
+      <c r="H36" s="13">
+        <f>H35-H34</f>
+        <v>1703936</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="13"/>
+        <v>208</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B6:B8 B10">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J14:L20">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+      <formula>"Y"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J27:K33">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
@@ -1407,10 +1861,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6:B8 B10 J14:L20" xr:uid="{EBA8029F-00D4-49E4-8B84-75C1EA9F44E8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6:B8 B10 J14:L20 J27:K33" xr:uid="{EBA8029F-00D4-49E4-8B84-75C1EA9F44E8}">
       <formula1>$B$1:$B$2</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Total size consumed cannot exceed total user flash size!" sqref="H21" xr:uid="{1D140836-F0E9-4E03-84AE-026A1CDC9976}">
+    <dataValidation type="decimal" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Total size consumed cannot exceed total user flash size!" sqref="H21 H34" xr:uid="{1D140836-F0E9-4E03-84AE-026A1CDC9976}">
       <formula1>H22</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
OEMiROT (NTZ): Update flash layout excel sheet
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H563ZI/Applications/ROT_NTZ/OEMiROT_NTZ_flash_layout.xlsx
+++ b/Projects/NUCLEO-H563ZI/Applications/ROT_NTZ/OEMiROT_NTZ_flash_layout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ST\Cube\Cube1\STM32CubeH5\Projects\NUCLEO-H563ZI\Applications\ROT_NTZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24400E7-1C51-415F-BDD4-B7C8C0861598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACF7692-412D-4964-915E-10E4F47E2774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{973ADE99-8809-4282-875C-44A8EA15E93C}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="160">
   <si>
     <t>offset</t>
   </si>
@@ -168,9 +168,6 @@
     <t>Source ref</t>
   </si>
   <si>
-    <t>stm32h563xx_flash.icf</t>
-  </si>
-  <si>
     <t>LOADER_CODE_SIZE</t>
   </si>
   <si>
@@ -213,9 +210,6 @@
     <t>OB flash &amp; provisioning script ext_loader flag</t>
   </si>
   <si>
-    <t>system_stm32h5xx.c</t>
-  </si>
-  <si>
     <t>VECT_TAB_OFFSET</t>
   </si>
   <si>
@@ -231,9 +225,6 @@
     <t>code size</t>
   </si>
   <si>
-    <t xml:space="preserve">Loader system init </t>
-  </si>
-  <si>
     <t>VTOR</t>
   </si>
   <si>
@@ -252,9 +243,6 @@
     <t>loaderaddress</t>
   </si>
   <si>
-    <t>Loader linker project</t>
-  </si>
-  <si>
     <t>img_config.bat</t>
   </si>
   <si>
@@ -270,10 +258,7 @@
     <t>Nb pages</t>
   </si>
   <si>
-    <t>wrpgrp1 loader start</t>
-  </si>
-  <si>
-    <t>wrpgrp1 loader end</t>
+    <t>wrpgrp1</t>
   </si>
   <si>
     <t>RE_LOADER_WRP_START</t>
@@ -304,13 +289,360 @@
   </si>
   <si>
     <t>App Download (Max)</t>
+  </si>
+  <si>
+    <t>RE_APP_IMAGE_NUMBER</t>
+  </si>
+  <si>
+    <t>RE_APP_DATA_IMAGE_NUMBER</t>
+  </si>
+  <si>
+    <t>app_image_number</t>
+  </si>
+  <si>
+    <t>app_data_image_number</t>
+  </si>
+  <si>
+    <t>RE_BL2_BOOT_ADDRESS</t>
+  </si>
+  <si>
+    <t>bootob, bootaddress</t>
+  </si>
+  <si>
+    <t>RE_BL2_WRP_START</t>
+  </si>
+  <si>
+    <t>RE_BL2_WRP_END</t>
+  </si>
+  <si>
+    <t>wrpgrp2</t>
+  </si>
+  <si>
+    <t>RE_BL2_HDP_START</t>
+  </si>
+  <si>
+    <t>RE_BL2_HDP_END</t>
+  </si>
+  <si>
+    <t>hdp</t>
+  </si>
+  <si>
+    <t>linker file</t>
+  </si>
+  <si>
+    <t>main.h</t>
+  </si>
+  <si>
+    <t>APP_CODE_OFFSET</t>
+  </si>
+  <si>
+    <t>RE_AREA_0_OFFSET</t>
+  </si>
+  <si>
+    <t>APP_CODE_SIZE</t>
+  </si>
+  <si>
+    <t>RE_IMAGE_FLASH_APP_IMAGE_SIZE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loader </t>
+  </si>
+  <si>
+    <t>Application</t>
+  </si>
+  <si>
+    <t>FW area size (-S option)</t>
+  </si>
+  <si>
+    <t>RE_ENCRYPTION</t>
+  </si>
+  <si>
+    <t>RE_OVER_WRITE</t>
+  </si>
+  <si>
+    <t>RE_FLASH_AREA_SCRATCH_SIZE</t>
+  </si>
+  <si>
+    <t>Encryption link</t>
+  </si>
+  <si>
+    <t>Write Option</t>
+  </si>
+  <si>
+    <t>Number of scratch sectors (-M option)</t>
+  </si>
+  <si>
+    <t>RE_IMAGE_FLASH_ADDRESS_APP</t>
+  </si>
+  <si>
+    <t>RE_IMAGE_FLASH_ADDRESS_DATA</t>
+  </si>
+  <si>
+    <t>RE_IMAGE_FLASH_DATA_IMAGE_SIZE</t>
+  </si>
+  <si>
+    <t>Data area size (-S option)</t>
+  </si>
+  <si>
+    <t>FW active area address</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">app code init xml (for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>init</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> hex image gen)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">app code xml (for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>update</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> binary image gen)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">data xml (for update </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>binary</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> image gen)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">data init xml (for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>init</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> hex image gen)</t>
+    </r>
+  </si>
+  <si>
+    <t>appli_flash_layout.h</t>
+  </si>
+  <si>
+    <t>MCUBOOT_OVERWRITE_ONLY</t>
+  </si>
+  <si>
+    <t>MCUBOOT_APP_IMAGE_NUMBER</t>
+  </si>
+  <si>
+    <t>MCUBOOT_S_DATA_IMAGE_NUMBER</t>
+  </si>
+  <si>
+    <t>RE_S_DATA_IMAGE_NUMBER</t>
+  </si>
+  <si>
+    <t>FLASH_AREA_0_OFFSET</t>
+  </si>
+  <si>
+    <t>FLASH_AREA_0_SIZE</t>
+  </si>
+  <si>
+    <t>RE_AREA_0_SIZE</t>
+  </si>
+  <si>
+    <t>FLASH_AREA_2_OFFSET</t>
+  </si>
+  <si>
+    <t>FLASH_AREA_2_SIZE</t>
+  </si>
+  <si>
+    <t>RE_AREA_2_OFFSET</t>
+  </si>
+  <si>
+    <t>RE_AREA_2_SIZE</t>
+  </si>
+  <si>
+    <t>FLASH_AREA_4_OFFSET</t>
+  </si>
+  <si>
+    <t>FLASH_AREA_4_SIZE</t>
+  </si>
+  <si>
+    <t>RE_AREA_4_OFFSET</t>
+  </si>
+  <si>
+    <t>RE_AREA_4_SIZE</t>
+  </si>
+  <si>
+    <t>FLASH_AREA_6_OFFSET</t>
+  </si>
+  <si>
+    <t>FLASH_AREA_6_SIZE</t>
+  </si>
+  <si>
+    <t>RE_AREA_6_OFFSET</t>
+  </si>
+  <si>
+    <t>RE_AREA_6_SIZE</t>
+  </si>
+  <si>
+    <t>FLASH_PARTITION_SIZE</t>
+  </si>
+  <si>
+    <t>FLASH_DATA_PARTITION_SIZE</t>
+  </si>
+  <si>
+    <t>FLASH_B_SIZE</t>
+  </si>
+  <si>
+    <t>RE_FLASH_B_SIZE</t>
+  </si>
+  <si>
+    <t>Loader main.h</t>
+  </si>
+  <si>
+    <t>App linker, App main.h, App app_flash_layout.h</t>
+  </si>
+  <si>
+    <t>App code init xml</t>
+  </si>
+  <si>
+    <t>Data init xml</t>
+  </si>
+  <si>
+    <t>loader main.h, App main.h, App linker, app code/init xml</t>
+  </si>
+  <si>
+    <t>data xml, data init xml</t>
+  </si>
+  <si>
+    <t>ob flash programming script</t>
+  </si>
+  <si>
+    <t>boot address ob, boot binary @</t>
+  </si>
+  <si>
+    <t>wrp for BL2</t>
+  </si>
+  <si>
+    <t>HDP for BL2</t>
+  </si>
+  <si>
+    <t>nb of app images</t>
+  </si>
+  <si>
+    <t>nb of data images</t>
+  </si>
+  <si>
+    <t>whether loader is used</t>
+  </si>
+  <si>
+    <t>App slot size</t>
+  </si>
+  <si>
+    <t>App active slot address</t>
+  </si>
+  <si>
+    <t>Data active slot address</t>
+  </si>
+  <si>
+    <t>Data slot size</t>
+  </si>
+  <si>
+    <t>Encryption support for update image</t>
+  </si>
+  <si>
+    <t>Overwrite only flag</t>
+  </si>
+  <si>
+    <t>App appli_flash_layout.h</t>
+  </si>
+  <si>
+    <t>Scratch area size</t>
+  </si>
+  <si>
+    <t>DATA image number</t>
+  </si>
+  <si>
+    <t>App download slot address</t>
+  </si>
+  <si>
+    <t>Data download slot address</t>
+  </si>
+  <si>
+    <t>Flash bank size</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -339,6 +671,51 @@
       <name val="Tahoma"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCE9178"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -360,7 +737,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -420,11 +797,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -433,6 +823,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -457,37 +848,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -503,14 +894,51 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -939,36 +1367,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="8">
         <v>8000000</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="8">
         <v>200000</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="8">
         <v>2000</v>
       </c>
     </row>
@@ -976,7 +1404,7 @@
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>6</v>
       </c>
     </row>
@@ -984,38 +1412,38 @@
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="5">
         <f>IF(($B$8="Y"),8000,0)</f>
         <v>8000</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>75</v>
-      </c>
-      <c r="B10" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1023,55 +1451,55 @@
       <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="6">
         <f>IF(($B$10="Y"),$B$5,0)</f>
         <v>2000</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="5"/>
+      <c r="B12" s="6"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" s="8" t="s">
+      <c r="E13" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="I13" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="J13" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="K13" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="L13" s="29"/>
+      <c r="I13" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="J13" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="K13" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="L13" s="30"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="11" t="s">
         <v>2</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -1088,7 +1516,7 @@
         <f>DEC2HEX(HEX2DEC(D14)+HEX2DEC(F14)-1)</f>
         <v>8017FFF</v>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="11">
         <v>18000</v>
       </c>
       <c r="G14" s="3">
@@ -1109,10 +1537,10 @@
       <c r="K14" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="L14" s="27"/>
+      <c r="L14" s="28"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="11" t="s">
         <v>8</v>
       </c>
       <c r="B15" s="3" t="s">
@@ -1152,10 +1580,10 @@
       <c r="K15" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="L15" s="27"/>
+      <c r="L15" s="28"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="11" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="3">
@@ -1195,11 +1623,11 @@
       <c r="K16" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="L16" s="27"/>
+      <c r="L16" s="28"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>78</v>
+      <c r="A17" s="11" t="s">
+        <v>73</v>
       </c>
       <c r="B17" s="3">
         <v>0</v>
@@ -1238,11 +1666,11 @@
       <c r="K17" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="L17" s="27"/>
+      <c r="L17" s="28"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
-        <v>79</v>
+      <c r="A18" s="11" t="s">
+        <v>74</v>
       </c>
       <c r="B18" s="3">
         <v>2</v>
@@ -1281,10 +1709,10 @@
       <c r="K18" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="L18" s="27"/>
+      <c r="L18" s="28"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="11" t="s">
         <v>15</v>
       </c>
       <c r="B19" s="3">
@@ -1324,10 +1752,10 @@
       <c r="K19" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="L19" s="27"/>
+      <c r="L19" s="28"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="11" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -1345,7 +1773,7 @@
         <f t="shared" si="0"/>
         <v>81FFFFF</v>
       </c>
-      <c r="F20" s="10">
+      <c r="F20" s="11">
         <f>$B$9</f>
         <v>8000</v>
       </c>
@@ -1367,7 +1795,7 @@
       <c r="K20" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="L20" s="27"/>
+      <c r="L20" s="28"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
@@ -1377,15 +1805,15 @@
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="12" t="str">
+      <c r="F21" s="13" t="str">
         <f>DEC2HEX(H21)</f>
         <v>200000</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21" s="5">
         <f t="shared" si="1"/>
         <v>2048</v>
       </c>
-      <c r="H21" s="13">
+      <c r="H21" s="14">
         <f>SUM(H14:H20)</f>
         <v>2097152</v>
       </c>
@@ -1395,21 +1823,21 @@
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="12" t="s">
         <v>22</v>
       </c>
       <c r="B22" t="s">
         <v>21</v>
       </c>
-      <c r="F22" s="13">
+      <c r="F22" s="14">
         <f>$B$4</f>
         <v>200000</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22" s="5">
         <f t="shared" si="1"/>
         <v>2048</v>
       </c>
-      <c r="H22" s="13">
+      <c r="H22" s="14">
         <f>HEX2DEC(F22)</f>
         <v>2097152</v>
       </c>
@@ -1419,18 +1847,18 @@
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="13" t="str">
+      <c r="F23" s="14" t="str">
         <f>DEC2HEX(H23)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23" s="5">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H23" s="13">
+      <c r="H23" s="14">
         <f>H22-H21</f>
         <v>0</v>
       </c>
@@ -1443,39 +1871,39 @@
       <c r="A26" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E26" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="F26" s="8" t="s">
+      <c r="E26" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="F26" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="8" t="s">
+      <c r="G26" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="I26" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="J26" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="K26" s="26" t="s">
-        <v>66</v>
+      <c r="I26" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="J26" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="K26" s="27" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="11" t="s">
         <v>2</v>
       </c>
       <c r="B27" s="3" t="s">
@@ -1492,7 +1920,7 @@
         <f>DEC2HEX(HEX2DEC(D27)+HEX2DEC(F27)-1)</f>
         <v>8017FFF</v>
       </c>
-      <c r="F27" s="10">
+      <c r="F27" s="11">
         <v>18000</v>
       </c>
       <c r="G27" s="3">
@@ -1515,7 +1943,7 @@
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="11" t="s">
         <v>8</v>
       </c>
       <c r="B28" s="3" t="s">
@@ -1557,7 +1985,7 @@
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="11" t="s">
         <v>14</v>
       </c>
       <c r="B29" s="3">
@@ -1599,7 +2027,7 @@
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B30" s="3">
@@ -1640,7 +2068,7 @@
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
+      <c r="A31" s="11" t="s">
         <v>13</v>
       </c>
       <c r="B31" s="3">
@@ -1682,7 +2110,7 @@
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="11" t="s">
         <v>15</v>
       </c>
       <c r="B32" s="3">
@@ -1724,7 +2152,7 @@
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="10" t="s">
+      <c r="A33" s="11" t="s">
         <v>10</v>
       </c>
       <c r="B33" s="3" t="s">
@@ -1742,7 +2170,7 @@
         <f t="shared" si="7"/>
         <v>805FFFF</v>
       </c>
-      <c r="F33" s="10">
+      <c r="F33" s="11">
         <f>$B$9</f>
         <v>8000</v>
       </c>
@@ -1773,15 +2201,15 @@
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
-      <c r="F34" s="12" t="str">
+      <c r="F34" s="13" t="str">
         <f>DEC2HEX(H34)</f>
         <v>60000</v>
       </c>
-      <c r="G34" s="4">
+      <c r="G34" s="5">
         <f t="shared" si="8"/>
         <v>384</v>
       </c>
-      <c r="H34" s="13">
+      <c r="H34" s="14">
         <f>SUM(H27:H33)</f>
         <v>393216</v>
       </c>
@@ -1791,21 +2219,21 @@
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="11" t="s">
+      <c r="A35" s="12" t="s">
         <v>22</v>
       </c>
       <c r="B35" t="s">
         <v>21</v>
       </c>
-      <c r="F35" s="13">
+      <c r="F35" s="14">
         <f>$B$4</f>
         <v>200000</v>
       </c>
-      <c r="G35" s="4">
+      <c r="G35" s="5">
         <f t="shared" si="8"/>
         <v>2048</v>
       </c>
-      <c r="H35" s="13">
+      <c r="H35" s="14">
         <f>HEX2DEC(F35)</f>
         <v>2097152</v>
       </c>
@@ -1815,18 +2243,18 @@
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="F36" s="13" t="str">
+      <c r="F36" s="14" t="str">
         <f>DEC2HEX(H36)</f>
         <v>1A0000</v>
       </c>
-      <c r="G36" s="4">
+      <c r="G36" s="5">
         <f t="shared" si="8"/>
         <v>1664</v>
       </c>
-      <c r="H36" s="13">
+      <c r="H36" s="14">
         <f>H35-H34</f>
         <v>1703936</v>
       </c>
@@ -1875,35 +2303,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EE97D97-B7AB-4B6E-A748-8501DA74A541}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="2.140625" customWidth="1"/>
     <col min="5" max="5" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E1" s="6" t="s">
+      <c r="A1" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="s">
         <v>37</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
       </c>
       <c r="E2" s="18" t="s">
         <v>29</v>
@@ -1920,211 +2349,856 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
         <v>39</v>
       </c>
-      <c r="B3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="F3" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="G3" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="H3" s="20" t="str">
+      <c r="E3" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="43" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" s="34" t="str">
         <f>A6</f>
         <v>RE_LOADER_CODE_START</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="A4" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="30"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="20" t="str">
+      <c r="C4" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="25"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="34" t="str">
         <f>A7</f>
         <v>RE_LOADER_CODE_SIZE</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="28" t="s">
-        <v>42</v>
+      <c r="A5" s="29" t="s">
+        <v>41</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>135</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E5" s="25"/>
-      <c r="F5" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="G5" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="H5" s="20" t="str">
+      <c r="F5" s="43" t="s">
+        <v>88</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="34" t="str">
         <f>A5</f>
         <v>RE_LOADER_CODE_OFFSET</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="28" t="s">
-        <v>44</v>
+      <c r="A6" s="29" t="s">
+        <v>43</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" s="20" t="s">
-        <v>68</v>
-      </c>
-      <c r="H6" s="20" t="str">
-        <f>A7</f>
-        <v>RE_LOADER_CODE_SIZE</v>
+        <v>55</v>
+      </c>
+      <c r="E6" s="25"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="H6" s="36" t="str">
+        <f>A14</f>
+        <v>RE_AREA_0_OFFSET</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
-        <v>52</v>
+      <c r="A7" s="29" t="s">
+        <v>50</v>
       </c>
       <c r="B7" t="s">
         <v>32</v>
       </c>
       <c r="C7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="26"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H7" s="42" t="str">
+        <f>A13</f>
+        <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="29" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" t="s">
         <v>54</v>
       </c>
-      <c r="E7" s="30"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="H7" s="20" t="str">
+      <c r="C8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="H8" s="34" t="str">
+        <f>A10</f>
+        <v>RE_LOADER</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="25"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="H9" s="36" t="str">
+        <f>A11</f>
+        <v>RE_APP_IMAGE_NUMBER</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" t="s">
+        <v>147</v>
+      </c>
+      <c r="E10" s="25"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="H10" s="36" t="str">
+        <f>A12</f>
+        <v>RE_APP_DATA_IMAGE_NUMBER</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="35" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" t="s">
+        <v>145</v>
+      </c>
+      <c r="E11" s="25"/>
+      <c r="F11" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="H11" s="38" t="str">
+        <f>A18</f>
+        <v>RE_BL2_BOOT_ADDRESS</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" t="s">
+        <v>146</v>
+      </c>
+      <c r="E12" s="25"/>
+      <c r="F12" s="45"/>
+      <c r="G12" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="H12" s="38" t="str">
+        <f>A19</f>
+        <v>RE_BL2_WRP_START</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" t="s">
+        <v>139</v>
+      </c>
+      <c r="C13" t="s">
+        <v>148</v>
+      </c>
+      <c r="E13" s="25"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="38" t="str">
+        <f>A20</f>
+        <v>RE_BL2_WRP_END</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C14" t="s">
+        <v>149</v>
+      </c>
+      <c r="E14" s="25"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="H14" s="34" t="str">
+        <f>A8</f>
+        <v>RE_LOADER_WRP_START</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" t="s">
+        <v>137</v>
+      </c>
+      <c r="C15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E15" s="25"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="34" t="str">
         <f>A9</f>
         <v>RE_LOADER_WRP_END</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E8" s="25"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="H8" s="20" t="str">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="B16" t="s">
+        <v>138</v>
+      </c>
+      <c r="C16" t="s">
+        <v>150</v>
+      </c>
+      <c r="E16" s="25"/>
+      <c r="F16" s="45"/>
+      <c r="G16" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="H16" s="38" t="str">
+        <f>A21</f>
+        <v>RE_BL2_HDP_START</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="46" t="s">
+        <v>104</v>
+      </c>
+      <c r="B17" t="s">
+        <v>140</v>
+      </c>
+      <c r="C17" t="s">
+        <v>151</v>
+      </c>
+      <c r="E17" s="25"/>
+      <c r="F17" s="45"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="39" t="str">
+        <f>A22</f>
+        <v>RE_BL2_HDP_END</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18" s="26"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H18" s="34" t="str">
         <f>A6</f>
         <v>RE_LOADER_CODE_START</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="28" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="G9" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="H9" s="20" t="str">
-        <f>A10</f>
-        <v>RE_LOADER</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-    </row>
-    <row r="17" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" t="s">
+        <v>141</v>
+      </c>
+      <c r="C19" t="s">
+        <v>143</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H19" s="36" t="str">
+        <f>A14</f>
+        <v>RE_AREA_0_OFFSET</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" t="s">
+        <v>141</v>
+      </c>
+      <c r="C20" t="s">
+        <v>143</v>
+      </c>
+      <c r="E20" s="25"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H20" s="42" t="str">
+        <f>A13</f>
+        <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" t="s">
+        <v>141</v>
+      </c>
+      <c r="C21" t="s">
+        <v>144</v>
+      </c>
+      <c r="E21" s="25"/>
+      <c r="F21" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H21" s="42" t="str">
+        <f>A13</f>
+        <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" t="s">
+        <v>141</v>
+      </c>
+      <c r="C22" t="s">
+        <v>144</v>
+      </c>
+      <c r="E22" s="25"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H22" s="2" t="str">
+        <f>A23</f>
+        <v>RE_ENCRYPTION</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" t="s">
+        <v>154</v>
+      </c>
+      <c r="C23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E23" s="25"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H23" s="2" t="str">
+        <f>A24</f>
+        <v>RE_OVER_WRITE</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" t="s">
+        <v>154</v>
+      </c>
+      <c r="C24" t="s">
+        <v>153</v>
+      </c>
+      <c r="E24" s="25"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H24" s="2" t="str">
+        <f>A25</f>
+        <v>RE_FLASH_AREA_SCRATCH_SIZE</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" t="s">
+        <v>155</v>
+      </c>
+      <c r="E25" s="25"/>
+      <c r="F25" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H25" s="42" t="str">
+        <f>A15</f>
+        <v>RE_IMAGE_FLASH_ADDRESS_APP</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="B26" t="s">
+        <v>154</v>
+      </c>
+      <c r="C26" t="s">
+        <v>156</v>
+      </c>
+      <c r="E26" s="25"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H26" s="42" t="str">
+        <f>A13</f>
+        <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" t="s">
+        <v>154</v>
+      </c>
+      <c r="C27" t="s">
+        <v>149</v>
+      </c>
+      <c r="E27" s="25"/>
+      <c r="F27" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H27" s="47" t="str">
+        <f>A17</f>
+        <v>RE_IMAGE_FLASH_DATA_IMAGE_SIZE</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="B28" t="s">
+        <v>154</v>
+      </c>
+      <c r="C28" t="s">
+        <v>148</v>
+      </c>
+      <c r="E28" s="25"/>
+      <c r="F28" s="48"/>
+      <c r="G28" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H28" s="2" t="str">
+        <f>A23</f>
+        <v>RE_ENCRYPTION</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" t="s">
+        <v>154</v>
+      </c>
+      <c r="C29" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" s="25"/>
+      <c r="F29" s="48"/>
+      <c r="G29" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H29" s="2" t="str">
+        <f>A24</f>
+        <v>RE_OVER_WRITE</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="B30" t="s">
+        <v>154</v>
+      </c>
+      <c r="C30" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="25"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H30" s="2" t="str">
+        <f>A25</f>
+        <v>RE_FLASH_AREA_SCRATCH_SIZE</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="B31" t="s">
+        <v>154</v>
+      </c>
+      <c r="C31" t="s">
+        <v>150</v>
+      </c>
+      <c r="E31" s="25"/>
+      <c r="F31" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H31" s="47" t="str">
+        <f>A16</f>
+        <v>RE_IMAGE_FLASH_ADDRESS_DATA</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="33" t="s">
+        <v>126</v>
+      </c>
+      <c r="B32" t="s">
+        <v>154</v>
+      </c>
+      <c r="C32" t="s">
+        <v>151</v>
+      </c>
+      <c r="E32" s="25"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H32" s="47" t="str">
+        <f>A17</f>
+        <v>RE_IMAGE_FLASH_DATA_IMAGE_SIZE</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="33" t="s">
+        <v>129</v>
+      </c>
+      <c r="B33" t="s">
+        <v>154</v>
+      </c>
+      <c r="C33" t="s">
+        <v>158</v>
+      </c>
+      <c r="E33" s="25"/>
+      <c r="F33" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H33" s="2" t="str">
+        <f>A14</f>
+        <v>RE_AREA_0_OFFSET</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="33" t="s">
+        <v>130</v>
+      </c>
+      <c r="B34" t="s">
+        <v>154</v>
+      </c>
+      <c r="C34" t="s">
+        <v>151</v>
+      </c>
+      <c r="E34" s="25"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H34" s="2" t="str">
+        <f>A13</f>
+        <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="B35" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" t="s">
+        <v>159</v>
+      </c>
+      <c r="E35" s="25"/>
+      <c r="F35" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H35" s="2" t="str">
+        <f>A24</f>
+        <v>RE_OVER_WRITE</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E36" s="25"/>
+      <c r="F36" s="48"/>
+      <c r="G36" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H36" s="2" t="str">
+        <f>A11</f>
+        <v>RE_APP_IMAGE_NUMBER</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E37" s="25"/>
+      <c r="F37" s="48"/>
+      <c r="G37" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H37" s="2" t="str">
+        <f>A26</f>
+        <v>RE_S_DATA_IMAGE_NUMBER</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E38" s="25"/>
+      <c r="F38" s="48"/>
+      <c r="G38" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="H38" s="2" t="str">
+        <f>A27</f>
+        <v>RE_AREA_0_OFFSET</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E39" s="25"/>
+      <c r="F39" s="48"/>
+      <c r="G39" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="H39" s="2" t="str">
+        <f>A28</f>
+        <v>RE_AREA_0_SIZE</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E40" s="25"/>
+      <c r="F40" s="48"/>
+      <c r="G40" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H40" s="2" t="str">
+        <f>A29</f>
+        <v>RE_AREA_2_OFFSET</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E41" s="25"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="H41" s="2" t="str">
+        <f>A30</f>
+        <v>RE_AREA_2_SIZE</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E42" s="25"/>
+      <c r="F42" s="48"/>
+      <c r="G42" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="H42" s="2" t="str">
+        <f>A31</f>
+        <v>RE_AREA_4_OFFSET</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E43" s="25"/>
+      <c r="F43" s="48"/>
+      <c r="G43" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H43" s="2" t="str">
+        <f>A32</f>
+        <v>RE_AREA_4_SIZE</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E44" s="25"/>
+      <c r="F44" s="48"/>
+      <c r="G44" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="H44" s="2" t="str">
+        <f>A33</f>
+        <v>RE_AREA_6_OFFSET</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E45" s="25"/>
+      <c r="F45" s="48"/>
+      <c r="G45" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="H45" s="2" t="str">
+        <f>A34</f>
+        <v>RE_AREA_6_SIZE</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E46" s="25"/>
+      <c r="F46" s="48"/>
+      <c r="G46" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="H46" s="42" t="str">
+        <f>A13</f>
+        <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E47" s="25"/>
+      <c r="F47" s="48"/>
+      <c r="G47" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="H47" s="47" t="str">
+        <f>A17</f>
+        <v>RE_IMAGE_FLASH_DATA_IMAGE_SIZE</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E48" s="25"/>
+      <c r="F48" s="48"/>
+      <c r="G48" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H48" s="41" t="str">
+        <f>A6</f>
+        <v>RE_LOADER_CODE_START</v>
+      </c>
+    </row>
+    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E49" s="26"/>
+      <c r="F49" s="23"/>
+      <c r="G49" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H49" s="2" t="str">
+        <f>A35</f>
+        <v>RE_FLASH_B_SIZE</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="17">
+    <mergeCell ref="F35:F49"/>
+    <mergeCell ref="E19:E49"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F21:F24"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="F27:F30"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="F11:F18"/>
+    <mergeCell ref="E8:E18"/>
+    <mergeCell ref="E3:E7"/>
+    <mergeCell ref="F5:F7"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="G12:G13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
OEMiROT (NTZ): Test flash layout with Primary only and add regression script
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H563ZI/Applications/ROT_NTZ/OEMiROT_NTZ_flash_layout.xlsx
+++ b/Projects/NUCLEO-H563ZI/Applications/ROT_NTZ/OEMiROT_NTZ_flash_layout.xlsx
@@ -8,14 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ST\Cube\Cube1\STM32CubeH5\Projects\NUCLEO-H563ZI\Applications\ROT_NTZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACF7692-412D-4964-915E-10E4F47E2774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E91070-8A6E-4E7C-B3A5-0E389C2D8964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{973ADE99-8809-4282-875C-44A8EA15E93C}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{973ADE99-8809-4282-875C-44A8EA15E93C}"/>
   </bookViews>
   <sheets>
     <sheet name="OEMiROT Flash Layout" sheetId="1" r:id="rId1"/>
     <sheet name="Build Actions" sheetId="2" r:id="rId2"/>
+    <sheet name="Test cases" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test cases'!$A$9:$L$34</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -64,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="185">
   <si>
     <t>offset</t>
   </si>
@@ -637,12 +641,87 @@
   <si>
     <t>Flash bank size</t>
   </si>
+  <si>
+    <t>Test case</t>
+  </si>
+  <si>
+    <t>EXT_LOADER</t>
+  </si>
+  <si>
+    <t>DATA_IMAGE_NUMBER</t>
+  </si>
+  <si>
+    <t>BOOT-&gt;Loader</t>
+  </si>
+  <si>
+    <t>BOOT-&gt;App</t>
+  </si>
+  <si>
+    <t>App-&gt;Loader</t>
+  </si>
+  <si>
+    <t>App Update</t>
+  </si>
+  <si>
+    <t>Data Update</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>ND</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>NOK</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>NT</t>
+  </si>
+  <si>
+    <t>Provisioning</t>
+  </si>
+  <si>
+    <t>IDE</t>
+  </si>
+  <si>
+    <t>IAR</t>
+  </si>
+  <si>
+    <t>KEIL</t>
+  </si>
+  <si>
+    <t>CubeIDE</t>
+  </si>
+  <si>
+    <t>Pre-step for each test cases:</t>
+  </si>
+  <si>
+    <t>Delete signed Data images in Provisioning Binary folder</t>
+  </si>
+  <si>
+    <t>Delete built materials of Boot, Loader, App in Binary folder</t>
+  </si>
+  <si>
+    <t>Clean projects in IDE</t>
+  </si>
+  <si>
+    <t>App confirm</t>
+  </si>
+  <si>
+    <t>Data confirm</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -664,12 +743,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -712,6 +785,21 @@
     <font>
       <sz val="11"/>
       <color theme="5" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -814,17 +902,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -835,11 +919,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -860,16 +943,48 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -884,67 +999,126 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="17">
+    <dxf>
+      <font>
+        <color theme="6"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0070C0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF00B0F0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1367,36 +1541,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="6">
         <v>8000000</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="6">
         <v>200000</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="6">
         <v>2000</v>
       </c>
     </row>
@@ -1404,7 +1578,7 @@
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1412,7 +1586,7 @@
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
@@ -1423,7 +1597,7 @@
       <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C8" t="s">
@@ -1434,7 +1608,7 @@
       <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="1">
         <f>IF(($B$8="Y"),8000,0)</f>
         <v>8000</v>
       </c>
@@ -1443,7 +1617,7 @@
       <c r="A10" t="s">
         <v>70</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="4" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1451,7 +1625,7 @@
       <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="4">
         <f>IF(($B$10="Y"),$B$5,0)</f>
         <v>2000</v>
       </c>
@@ -1460,46 +1634,46 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="6"/>
+      <c r="B12" s="4"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="J13" s="27" t="s">
+      <c r="J13" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="K13" s="27" t="s">
+      <c r="K13" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="L13" s="30"/>
+      <c r="L13" s="6"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="8" t="s">
         <v>2</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -1516,7 +1690,7 @@
         <f>DEC2HEX(HEX2DEC(D14)+HEX2DEC(F14)-1)</f>
         <v>8017FFF</v>
       </c>
-      <c r="F14" s="11">
+      <c r="F14" s="8">
         <v>18000</v>
       </c>
       <c r="G14" s="3">
@@ -1527,20 +1701,20 @@
         <f>HEX2DEC(F14)</f>
         <v>98304</v>
       </c>
-      <c r="I14" s="17">
+      <c r="I14" s="14">
         <f>H14/HEX2DEC($B$5)</f>
         <v>12</v>
       </c>
-      <c r="J14" s="17" t="s">
+      <c r="J14" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K14" s="17" t="s">
+      <c r="K14" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="L14" s="28"/>
+      <c r="L14" s="4"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="8" t="s">
         <v>8</v>
       </c>
       <c r="B15" s="3" t="s">
@@ -1570,20 +1744,20 @@
         <f t="shared" ref="H15:H19" si="2">HEX2DEC(F15)</f>
         <v>65536</v>
       </c>
-      <c r="I15" s="17">
+      <c r="I15" s="14">
         <f t="shared" ref="I15:I19" si="3">H15/HEX2DEC($B$5)</f>
         <v>8</v>
       </c>
-      <c r="J15" s="17" t="s">
+      <c r="J15" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K15" s="17" t="s">
+      <c r="K15" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="L15" s="28"/>
+      <c r="L15" s="4"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="8" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="3">
@@ -1613,20 +1787,20 @@
         <f t="shared" si="2"/>
         <v>8192</v>
       </c>
-      <c r="I16" s="17">
+      <c r="I16" s="14">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="J16" s="17" t="s">
+      <c r="J16" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K16" s="17" t="s">
+      <c r="K16" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="L16" s="28"/>
+      <c r="L16" s="4"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="8" t="s">
         <v>73</v>
       </c>
       <c r="B17" s="3">
@@ -1644,7 +1818,7 @@
         <f t="shared" si="0"/>
         <v>810FFFF</v>
       </c>
-      <c r="F17" s="31" t="str">
+      <c r="F17" s="18" t="str">
         <f>DEC2HEX(IF($B$6="N",ROUNDDOWN((HEX2DEC(B4)-HEX2DEC(F14)-HEX2DEC(F15)-HEX2DEC(F20)-HEX2DEC(F16)-HEX2DEC(F19))/2/HEX2DEC($B$5),0)*HEX2DEC($B$5),(HEX2DEC(B4)-HEX2DEC(F14)-HEX2DEC(F15)-HEX2DEC(F20)-HEX2DEC(F16)-HEX2DEC(F19))))</f>
         <v>E6000</v>
       </c>
@@ -1656,20 +1830,20 @@
         <f t="shared" si="2"/>
         <v>942080</v>
       </c>
-      <c r="I17" s="17">
+      <c r="I17" s="14">
         <f t="shared" si="3"/>
         <v>115</v>
       </c>
-      <c r="J17" s="17" t="s">
+      <c r="J17" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K17" s="17" t="s">
+      <c r="K17" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="L17" s="28"/>
+      <c r="L17" s="4"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="8" t="s">
         <v>74</v>
       </c>
       <c r="B18" s="3">
@@ -1687,7 +1861,7 @@
         <f t="shared" si="0"/>
         <v>81F5FFF</v>
       </c>
-      <c r="F18" s="31" t="str">
+      <c r="F18" s="18" t="str">
         <f>IF($B$6="N",F17,0)</f>
         <v>E6000</v>
       </c>
@@ -1699,20 +1873,20 @@
         <f t="shared" si="2"/>
         <v>942080</v>
       </c>
-      <c r="I18" s="17">
+      <c r="I18" s="14">
         <f t="shared" si="3"/>
         <v>115</v>
       </c>
-      <c r="J18" s="17" t="s">
+      <c r="J18" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K18" s="17" t="s">
+      <c r="K18" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="L18" s="28"/>
+      <c r="L18" s="4"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="8" t="s">
         <v>15</v>
       </c>
       <c r="B19" s="3">
@@ -1742,20 +1916,20 @@
         <f t="shared" si="2"/>
         <v>8192</v>
       </c>
-      <c r="I19" s="17">
+      <c r="I19" s="14">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="J19" s="17" t="s">
+      <c r="J19" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K19" s="17" t="s">
+      <c r="K19" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="L19" s="28"/>
+      <c r="L19" s="4"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="8" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -1773,7 +1947,7 @@
         <f t="shared" si="0"/>
         <v>81FFFFF</v>
       </c>
-      <c r="F20" s="11">
+      <c r="F20" s="8">
         <f>$B$9</f>
         <v>8000</v>
       </c>
@@ -1785,17 +1959,17 @@
         <f>HEX2DEC(F20)</f>
         <v>32768</v>
       </c>
-      <c r="I20" s="17">
+      <c r="I20" s="14">
         <f>H20/HEX2DEC($B$5)</f>
         <v>4</v>
       </c>
-      <c r="J20" s="17" t="s">
+      <c r="J20" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K20" s="17" t="s">
+      <c r="K20" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="L20" s="28"/>
+      <c r="L20" s="4"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
@@ -1805,15 +1979,15 @@
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="13" t="str">
+      <c r="F21" s="10" t="str">
         <f>DEC2HEX(H21)</f>
         <v>200000</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="1">
         <f t="shared" si="1"/>
         <v>2048</v>
       </c>
-      <c r="H21" s="14">
+      <c r="H21" s="11">
         <f>SUM(H14:H20)</f>
         <v>2097152</v>
       </c>
@@ -1823,21 +1997,21 @@
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B22" t="s">
         <v>21</v>
       </c>
-      <c r="F22" s="14">
+      <c r="F22" s="11">
         <f>$B$4</f>
         <v>200000</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="1">
         <f t="shared" si="1"/>
         <v>2048</v>
       </c>
-      <c r="H22" s="14">
+      <c r="H22" s="11">
         <f>HEX2DEC(F22)</f>
         <v>2097152</v>
       </c>
@@ -1847,18 +2021,18 @@
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="14" t="str">
+      <c r="F23" s="11" t="str">
         <f>DEC2HEX(H23)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H23" s="14">
+      <c r="H23" s="11">
         <f>H22-H21</f>
         <v>0</v>
       </c>
@@ -1868,42 +2042,42 @@
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
+      <c r="A26" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G26" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H26" s="10" t="s">
+      <c r="H26" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="I26" s="10" t="s">
+      <c r="I26" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="J26" s="27" t="s">
+      <c r="J26" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="K26" s="27" t="s">
+      <c r="K26" s="12" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="8" t="s">
         <v>2</v>
       </c>
       <c r="B27" s="3" t="s">
@@ -1920,7 +2094,7 @@
         <f>DEC2HEX(HEX2DEC(D27)+HEX2DEC(F27)-1)</f>
         <v>8017FFF</v>
       </c>
-      <c r="F27" s="11">
+      <c r="F27" s="8">
         <v>18000</v>
       </c>
       <c r="G27" s="3">
@@ -1931,19 +2105,19 @@
         <f>HEX2DEC(F27)</f>
         <v>98304</v>
       </c>
-      <c r="I27" s="17">
+      <c r="I27" s="14">
         <f>H27/HEX2DEC($B$5)</f>
         <v>12</v>
       </c>
-      <c r="J27" s="17" t="s">
+      <c r="J27" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K27" s="17" t="s">
+      <c r="K27" s="14" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="8" t="s">
         <v>8</v>
       </c>
       <c r="B28" s="3" t="s">
@@ -1973,19 +2147,19 @@
         <f t="shared" ref="H28:H32" si="9">HEX2DEC(F28)</f>
         <v>65536</v>
       </c>
-      <c r="I28" s="17">
+      <c r="I28" s="14">
         <f t="shared" ref="I28:I32" si="10">H28/HEX2DEC($B$5)</f>
         <v>8</v>
       </c>
-      <c r="J28" s="17" t="s">
+      <c r="J28" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K28" s="17" t="s">
+      <c r="K28" s="14" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="8" t="s">
         <v>14</v>
       </c>
       <c r="B29" s="3">
@@ -2015,19 +2189,19 @@
         <f t="shared" si="9"/>
         <v>8192</v>
       </c>
-      <c r="I29" s="17">
+      <c r="I29" s="14">
         <f t="shared" si="10"/>
         <v>1</v>
       </c>
-      <c r="J29" s="17" t="s">
+      <c r="J29" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K29" s="17" t="s">
+      <c r="K29" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="8" t="s">
         <v>12</v>
       </c>
       <c r="B30" s="3">
@@ -2045,7 +2219,7 @@
         <f t="shared" si="7"/>
         <v>803FFFF</v>
       </c>
-      <c r="F30" s="32">
+      <c r="F30" s="19">
         <v>16000</v>
       </c>
       <c r="G30" s="3">
@@ -2056,19 +2230,19 @@
         <f t="shared" si="9"/>
         <v>90112</v>
       </c>
-      <c r="I30" s="17">
+      <c r="I30" s="14">
         <f t="shared" si="10"/>
         <v>11</v>
       </c>
-      <c r="J30" s="17" t="s">
+      <c r="J30" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K30" s="17" t="s">
+      <c r="K30" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B31" s="3">
@@ -2086,7 +2260,7 @@
         <f t="shared" si="7"/>
         <v>8055FFF</v>
       </c>
-      <c r="F31" s="32">
+      <c r="F31" s="19">
         <f>IF($B$6="N",F30,0)</f>
         <v>16000</v>
       </c>
@@ -2098,19 +2272,19 @@
         <f t="shared" si="9"/>
         <v>90112</v>
       </c>
-      <c r="I31" s="17">
+      <c r="I31" s="14">
         <f t="shared" si="10"/>
         <v>11</v>
       </c>
-      <c r="J31" s="17" t="s">
+      <c r="J31" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K31" s="17" t="s">
+      <c r="K31" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="8" t="s">
         <v>15</v>
       </c>
       <c r="B32" s="3">
@@ -2140,19 +2314,19 @@
         <f t="shared" si="9"/>
         <v>8192</v>
       </c>
-      <c r="I32" s="17">
+      <c r="I32" s="14">
         <f t="shared" si="10"/>
         <v>1</v>
       </c>
-      <c r="J32" s="17" t="s">
+      <c r="J32" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="K32" s="17" t="s">
+      <c r="K32" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="8" t="s">
         <v>10</v>
       </c>
       <c r="B33" s="3" t="s">
@@ -2170,7 +2344,7 @@
         <f t="shared" si="7"/>
         <v>805FFFF</v>
       </c>
-      <c r="F33" s="11">
+      <c r="F33" s="8">
         <f>$B$9</f>
         <v>8000</v>
       </c>
@@ -2182,14 +2356,14 @@
         <f>HEX2DEC(F33)</f>
         <v>32768</v>
       </c>
-      <c r="I33" s="17">
+      <c r="I33" s="14">
         <f>H33/HEX2DEC($B$5)</f>
         <v>4</v>
       </c>
-      <c r="J33" s="17" t="s">
+      <c r="J33" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K33" s="17" t="s">
+      <c r="K33" s="14" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2201,15 +2375,15 @@
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
-      <c r="F34" s="13" t="str">
+      <c r="F34" s="10" t="str">
         <f>DEC2HEX(H34)</f>
         <v>60000</v>
       </c>
-      <c r="G34" s="5">
+      <c r="G34" s="1">
         <f t="shared" si="8"/>
         <v>384</v>
       </c>
-      <c r="H34" s="14">
+      <c r="H34" s="11">
         <f>SUM(H27:H33)</f>
         <v>393216</v>
       </c>
@@ -2219,21 +2393,21 @@
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B35" t="s">
         <v>21</v>
       </c>
-      <c r="F35" s="14">
+      <c r="F35" s="11">
         <f>$B$4</f>
         <v>200000</v>
       </c>
-      <c r="G35" s="5">
+      <c r="G35" s="1">
         <f t="shared" si="8"/>
         <v>2048</v>
       </c>
-      <c r="H35" s="14">
+      <c r="H35" s="11">
         <f>HEX2DEC(F35)</f>
         <v>2097152</v>
       </c>
@@ -2243,18 +2417,18 @@
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F36" s="14" t="str">
+      <c r="F36" s="11" t="str">
         <f>DEC2HEX(H36)</f>
         <v>1A0000</v>
       </c>
-      <c r="G36" s="5">
+      <c r="G36" s="1">
         <f t="shared" si="8"/>
         <v>1664</v>
       </c>
-      <c r="H36" s="14">
+      <c r="H36" s="11">
         <f>H35-H34</f>
         <v>1703936</v>
       </c>
@@ -2265,26 +2439,26 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:B8 B10">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="5" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="6" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J14:L20">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+  <conditionalFormatting sqref="J27:K33">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J27:K33">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="J14:L20">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
       <formula>"N"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="4" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2320,10 +2494,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2334,16 +2508,16 @@
       <c r="B2" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="15" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2354,42 +2528,42 @@
       <c r="B3" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="35" t="s">
         <v>93</v>
       </c>
-      <c r="F3" s="43" t="s">
+      <c r="F3" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="H3" s="34" t="str">
+      <c r="H3" s="21" t="str">
         <f>A6</f>
         <v>RE_LOADER_CODE_START</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="25"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="22" t="s">
+      <c r="E4" s="36"/>
+      <c r="F4" s="42"/>
+      <c r="G4" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="34" t="str">
+      <c r="H4" s="21" t="str">
         <f>A7</f>
         <v>RE_LOADER_CODE_SIZE</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="17" t="s">
         <v>41</v>
       </c>
       <c r="B5" t="s">
@@ -2398,40 +2572,40 @@
       <c r="C5" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="25"/>
-      <c r="F5" s="43" t="s">
+      <c r="E5" s="36"/>
+      <c r="F5" s="40" t="s">
         <v>88</v>
       </c>
-      <c r="G5" s="22" t="s">
+      <c r="G5" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="H5" s="34" t="str">
+      <c r="H5" s="21" t="str">
         <f>A5</f>
         <v>RE_LOADER_CODE_OFFSET</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="13" t="s">
         <v>51</v>
       </c>
       <c r="C6" t="s">
         <v>55</v>
       </c>
-      <c r="E6" s="25"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="22" t="s">
+      <c r="E6" s="36"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="H6" s="36" t="str">
+      <c r="H6" s="23" t="str">
         <f>A14</f>
         <v>RE_AREA_0_OFFSET</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="17" t="s">
         <v>50</v>
       </c>
       <c r="B7" t="s">
@@ -2440,18 +2614,18 @@
       <c r="C7" t="s">
         <v>52</v>
       </c>
-      <c r="E7" s="26"/>
-      <c r="F7" s="44"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="42"/>
       <c r="G7" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H7" s="42" t="str">
+      <c r="H7" s="29" t="str">
         <f>A13</f>
         <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="17" t="s">
         <v>65</v>
       </c>
       <c r="B8" t="s">
@@ -2460,22 +2634,22 @@
       <c r="C8" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="43" t="s">
+      <c r="F8" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="G8" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="H8" s="34" t="str">
+      <c r="H8" s="21" t="str">
         <f>A10</f>
         <v>RE_LOADER</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="17" t="s">
         <v>42</v>
       </c>
       <c r="B9" t="s">
@@ -2484,18 +2658,18 @@
       <c r="C9" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="25"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="22" t="s">
+      <c r="E9" s="36"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="36" t="str">
+      <c r="H9" s="23" t="str">
         <f>A11</f>
         <v>RE_APP_IMAGE_NUMBER</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="17" t="s">
         <v>44</v>
       </c>
       <c r="B10" t="s">
@@ -2504,18 +2678,18 @@
       <c r="C10" t="s">
         <v>147</v>
       </c>
-      <c r="E10" s="25"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="22" t="s">
+      <c r="E10" s="36"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="36" t="str">
+      <c r="H10" s="23" t="str">
         <f>A12</f>
         <v>RE_APP_DATA_IMAGE_NUMBER</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="35" t="s">
+      <c r="A11" s="22" t="s">
         <v>75</v>
       </c>
       <c r="B11" t="s">
@@ -2524,20 +2698,20 @@
       <c r="C11" t="s">
         <v>145</v>
       </c>
-      <c r="E11" s="25"/>
-      <c r="F11" s="43" t="s">
+      <c r="E11" s="36"/>
+      <c r="F11" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="22" t="s">
+      <c r="G11" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="38" t="str">
+      <c r="H11" s="25" t="str">
         <f>A18</f>
         <v>RE_BL2_BOOT_ADDRESS</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="22" t="s">
         <v>76</v>
       </c>
       <c r="B12" t="s">
@@ -2546,18 +2720,18 @@
       <c r="C12" t="s">
         <v>146</v>
       </c>
-      <c r="E12" s="25"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="21" t="s">
+      <c r="E12" s="36"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="H12" s="38" t="str">
+      <c r="H12" s="25" t="str">
         <f>A19</f>
         <v>RE_BL2_WRP_START</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="35" t="s">
+      <c r="A13" s="22" t="s">
         <v>92</v>
       </c>
       <c r="B13" t="s">
@@ -2566,16 +2740,16 @@
       <c r="C13" t="s">
         <v>148</v>
       </c>
-      <c r="E13" s="25"/>
-      <c r="F13" s="45"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="38" t="str">
+      <c r="E13" s="36"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="25" t="str">
         <f>A20</f>
         <v>RE_BL2_WRP_END</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="35" t="s">
+      <c r="A14" s="22" t="s">
         <v>90</v>
       </c>
       <c r="B14" t="s">
@@ -2584,18 +2758,18 @@
       <c r="C14" t="s">
         <v>149</v>
       </c>
-      <c r="E14" s="25"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="21" t="s">
+      <c r="E14" s="36"/>
+      <c r="F14" s="41"/>
+      <c r="G14" s="32" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="34" t="str">
+      <c r="H14" s="21" t="str">
         <f>A8</f>
         <v>RE_LOADER_WRP_START</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="35" t="s">
+      <c r="A15" s="22" t="s">
         <v>102</v>
       </c>
       <c r="B15" t="s">
@@ -2604,16 +2778,16 @@
       <c r="C15" t="s">
         <v>149</v>
       </c>
-      <c r="E15" s="25"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="34" t="str">
+      <c r="E15" s="36"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="21" t="str">
         <f>A9</f>
         <v>RE_LOADER_WRP_END</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="46" t="s">
+      <c r="A16" s="30" t="s">
         <v>103</v>
       </c>
       <c r="B16" t="s">
@@ -2622,18 +2796,18 @@
       <c r="C16" t="s">
         <v>150</v>
       </c>
-      <c r="E16" s="25"/>
-      <c r="F16" s="45"/>
-      <c r="G16" s="21" t="s">
+      <c r="E16" s="36"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="32" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="38" t="str">
+      <c r="H16" s="25" t="str">
         <f>A21</f>
         <v>RE_BL2_HDP_START</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="46" t="s">
+      <c r="A17" s="30" t="s">
         <v>104</v>
       </c>
       <c r="B17" t="s">
@@ -2642,16 +2816,16 @@
       <c r="C17" t="s">
         <v>151</v>
       </c>
-      <c r="E17" s="25"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="39" t="str">
+      <c r="E17" s="36"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="26" t="str">
         <f>A22</f>
         <v>RE_BL2_HDP_END</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="37" t="s">
+      <c r="A18" s="24" t="s">
         <v>79</v>
       </c>
       <c r="B18" t="s">
@@ -2660,18 +2834,18 @@
       <c r="C18" t="s">
         <v>142</v>
       </c>
-      <c r="E18" s="26"/>
-      <c r="F18" s="44"/>
-      <c r="G18" s="40" t="s">
+      <c r="E18" s="37"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="H18" s="34" t="str">
+      <c r="H18" s="21" t="str">
         <f>A6</f>
         <v>RE_LOADER_CODE_START</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="37" t="s">
+      <c r="A19" s="24" t="s">
         <v>81</v>
       </c>
       <c r="B19" t="s">
@@ -2680,22 +2854,22 @@
       <c r="C19" t="s">
         <v>143</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="F19" s="21" t="s">
+      <c r="F19" s="32" t="s">
         <v>87</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="H19" s="36" t="str">
+      <c r="H19" s="23" t="str">
         <f>A14</f>
         <v>RE_AREA_0_OFFSET</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="37" t="s">
+      <c r="A20" s="24" t="s">
         <v>82</v>
       </c>
       <c r="B20" t="s">
@@ -2704,18 +2878,18 @@
       <c r="C20" t="s">
         <v>143</v>
       </c>
-      <c r="E20" s="25"/>
-      <c r="F20" s="23"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="34"/>
       <c r="G20" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="42" t="str">
+      <c r="H20" s="29" t="str">
         <f>A13</f>
         <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="24" t="s">
         <v>84</v>
       </c>
       <c r="B21" t="s">
@@ -2724,20 +2898,20 @@
       <c r="C21" t="s">
         <v>144</v>
       </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="21" t="s">
+      <c r="E21" s="36"/>
+      <c r="F21" s="32" t="s">
         <v>108</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="H21" s="42" t="str">
+      <c r="H21" s="29" t="str">
         <f>A13</f>
         <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="24" t="s">
         <v>85</v>
       </c>
       <c r="B22" t="s">
@@ -2746,8 +2920,8 @@
       <c r="C22" t="s">
         <v>144</v>
       </c>
-      <c r="E22" s="25"/>
-      <c r="F22" s="48"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="33"/>
       <c r="G22" s="2" t="s">
         <v>99</v>
       </c>
@@ -2757,7 +2931,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="33" t="s">
+      <c r="A23" s="20" t="s">
         <v>96</v>
       </c>
       <c r="B23" t="s">
@@ -2766,8 +2940,8 @@
       <c r="C23" t="s">
         <v>152</v>
       </c>
-      <c r="E23" s="25"/>
-      <c r="F23" s="48"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="33"/>
       <c r="G23" s="2" t="s">
         <v>100</v>
       </c>
@@ -2777,7 +2951,7 @@
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="33" t="s">
+      <c r="A24" s="20" t="s">
         <v>97</v>
       </c>
       <c r="B24" t="s">
@@ -2786,8 +2960,8 @@
       <c r="C24" t="s">
         <v>153</v>
       </c>
-      <c r="E24" s="25"/>
-      <c r="F24" s="23"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="34"/>
       <c r="G24" s="2" t="s">
         <v>101</v>
       </c>
@@ -2797,7 +2971,7 @@
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="33" t="s">
+      <c r="A25" s="20" t="s">
         <v>98</v>
       </c>
       <c r="B25" t="s">
@@ -2806,20 +2980,20 @@
       <c r="C25" t="s">
         <v>155</v>
       </c>
-      <c r="E25" s="25"/>
-      <c r="F25" s="21" t="s">
+      <c r="E25" s="36"/>
+      <c r="F25" s="32" t="s">
         <v>107</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="H25" s="42" t="str">
+      <c r="H25" s="29" t="str">
         <f>A15</f>
         <v>RE_IMAGE_FLASH_ADDRESS_APP</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="20" t="s">
         <v>115</v>
       </c>
       <c r="B26" t="s">
@@ -2828,18 +3002,18 @@
       <c r="C26" t="s">
         <v>156</v>
       </c>
-      <c r="E26" s="25"/>
-      <c r="F26" s="23"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="34"/>
       <c r="G26" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="H26" s="42" t="str">
+      <c r="H26" s="29" t="str">
         <f>A13</f>
         <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="33" t="s">
+      <c r="A27" s="20" t="s">
         <v>90</v>
       </c>
       <c r="B27" t="s">
@@ -2848,20 +3022,20 @@
       <c r="C27" t="s">
         <v>149</v>
       </c>
-      <c r="E27" s="25"/>
-      <c r="F27" s="21" t="s">
+      <c r="E27" s="36"/>
+      <c r="F27" s="32" t="s">
         <v>109</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H27" s="47" t="str">
+      <c r="H27" s="31" t="str">
         <f>A17</f>
         <v>RE_IMAGE_FLASH_DATA_IMAGE_SIZE</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="33" t="s">
+      <c r="A28" s="20" t="s">
         <v>118</v>
       </c>
       <c r="B28" t="s">
@@ -2870,8 +3044,8 @@
       <c r="C28" t="s">
         <v>148</v>
       </c>
-      <c r="E28" s="25"/>
-      <c r="F28" s="48"/>
+      <c r="E28" s="36"/>
+      <c r="F28" s="33"/>
       <c r="G28" s="2" t="s">
         <v>99</v>
       </c>
@@ -2881,7 +3055,7 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="33" t="s">
+      <c r="A29" s="20" t="s">
         <v>121</v>
       </c>
       <c r="B29" t="s">
@@ -2890,8 +3064,8 @@
       <c r="C29" t="s">
         <v>157</v>
       </c>
-      <c r="E29" s="25"/>
-      <c r="F29" s="48"/>
+      <c r="E29" s="36"/>
+      <c r="F29" s="33"/>
       <c r="G29" s="2" t="s">
         <v>100</v>
       </c>
@@ -2901,7 +3075,7 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="33" t="s">
+      <c r="A30" s="20" t="s">
         <v>122</v>
       </c>
       <c r="B30" t="s">
@@ -2910,8 +3084,8 @@
       <c r="C30" t="s">
         <v>148</v>
       </c>
-      <c r="E30" s="25"/>
-      <c r="F30" s="23"/>
+      <c r="E30" s="36"/>
+      <c r="F30" s="34"/>
       <c r="G30" s="2" t="s">
         <v>101</v>
       </c>
@@ -2921,7 +3095,7 @@
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="33" t="s">
+      <c r="A31" s="20" t="s">
         <v>125</v>
       </c>
       <c r="B31" t="s">
@@ -2930,20 +3104,20 @@
       <c r="C31" t="s">
         <v>150</v>
       </c>
-      <c r="E31" s="25"/>
-      <c r="F31" s="21" t="s">
+      <c r="E31" s="36"/>
+      <c r="F31" s="32" t="s">
         <v>110</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="H31" s="47" t="str">
+      <c r="H31" s="31" t="str">
         <f>A16</f>
         <v>RE_IMAGE_FLASH_ADDRESS_DATA</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="33" t="s">
+      <c r="A32" s="20" t="s">
         <v>126</v>
       </c>
       <c r="B32" t="s">
@@ -2952,18 +3126,18 @@
       <c r="C32" t="s">
         <v>151</v>
       </c>
-      <c r="E32" s="25"/>
-      <c r="F32" s="23"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="34"/>
       <c r="G32" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="H32" s="47" t="str">
+      <c r="H32" s="31" t="str">
         <f>A17</f>
         <v>RE_IMAGE_FLASH_DATA_IMAGE_SIZE</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="20" t="s">
         <v>129</v>
       </c>
       <c r="B33" t="s">
@@ -2972,8 +3146,8 @@
       <c r="C33" t="s">
         <v>158</v>
       </c>
-      <c r="E33" s="25"/>
-      <c r="F33" s="19" t="s">
+      <c r="E33" s="36"/>
+      <c r="F33" s="38" t="s">
         <v>88</v>
       </c>
       <c r="G33" s="2" t="s">
@@ -2985,7 +3159,7 @@
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="33" t="s">
+      <c r="A34" s="20" t="s">
         <v>130</v>
       </c>
       <c r="B34" t="s">
@@ -2994,8 +3168,8 @@
       <c r="C34" t="s">
         <v>151</v>
       </c>
-      <c r="E34" s="25"/>
-      <c r="F34" s="20"/>
+      <c r="E34" s="36"/>
+      <c r="F34" s="39"/>
       <c r="G34" s="2" t="s">
         <v>91</v>
       </c>
@@ -3005,7 +3179,7 @@
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="33" t="s">
+      <c r="A35" s="20" t="s">
         <v>134</v>
       </c>
       <c r="B35" t="s">
@@ -3014,8 +3188,8 @@
       <c r="C35" t="s">
         <v>159</v>
       </c>
-      <c r="E35" s="25"/>
-      <c r="F35" s="21" t="s">
+      <c r="E35" s="36"/>
+      <c r="F35" s="32" t="s">
         <v>111</v>
       </c>
       <c r="G35" s="2" t="s">
@@ -3027,8 +3201,8 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E36" s="25"/>
-      <c r="F36" s="48"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="33"/>
       <c r="G36" s="2" t="s">
         <v>113</v>
       </c>
@@ -3038,141 +3212,141 @@
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E37" s="25"/>
-      <c r="F37" s="48"/>
+      <c r="E37" s="36"/>
+      <c r="F37" s="33"/>
       <c r="G37" s="2" t="s">
         <v>114</v>
       </c>
       <c r="H37" s="2" t="str">
-        <f>A26</f>
+        <f t="shared" ref="H37:H45" si="0">A26</f>
         <v>RE_S_DATA_IMAGE_NUMBER</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E38" s="25"/>
-      <c r="F38" s="48"/>
-      <c r="G38" s="4" t="s">
+      <c r="E38" s="36"/>
+      <c r="F38" s="33"/>
+      <c r="G38" s="2" t="s">
         <v>116</v>
       </c>
       <c r="H38" s="2" t="str">
-        <f>A27</f>
+        <f t="shared" si="0"/>
         <v>RE_AREA_0_OFFSET</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E39" s="25"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="4" t="s">
+      <c r="E39" s="36"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="2" t="s">
         <v>117</v>
       </c>
       <c r="H39" s="2" t="str">
-        <f>A28</f>
+        <f t="shared" si="0"/>
         <v>RE_AREA_0_SIZE</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E40" s="25"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="4" t="s">
+      <c r="E40" s="36"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="2" t="s">
         <v>119</v>
       </c>
       <c r="H40" s="2" t="str">
-        <f>A29</f>
+        <f t="shared" si="0"/>
         <v>RE_AREA_2_OFFSET</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E41" s="25"/>
-      <c r="F41" s="48"/>
-      <c r="G41" s="4" t="s">
+      <c r="E41" s="36"/>
+      <c r="F41" s="33"/>
+      <c r="G41" s="2" t="s">
         <v>120</v>
       </c>
       <c r="H41" s="2" t="str">
-        <f>A30</f>
+        <f t="shared" si="0"/>
         <v>RE_AREA_2_SIZE</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E42" s="25"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="4" t="s">
+      <c r="E42" s="36"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="2" t="s">
         <v>123</v>
       </c>
       <c r="H42" s="2" t="str">
-        <f>A31</f>
+        <f t="shared" si="0"/>
         <v>RE_AREA_4_OFFSET</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E43" s="25"/>
-      <c r="F43" s="48"/>
-      <c r="G43" s="4" t="s">
+      <c r="E43" s="36"/>
+      <c r="F43" s="33"/>
+      <c r="G43" s="2" t="s">
         <v>124</v>
       </c>
       <c r="H43" s="2" t="str">
-        <f>A32</f>
+        <f t="shared" si="0"/>
         <v>RE_AREA_4_SIZE</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E44" s="25"/>
-      <c r="F44" s="48"/>
-      <c r="G44" s="4" t="s">
+      <c r="E44" s="36"/>
+      <c r="F44" s="33"/>
+      <c r="G44" s="2" t="s">
         <v>127</v>
       </c>
       <c r="H44" s="2" t="str">
-        <f>A33</f>
+        <f t="shared" si="0"/>
         <v>RE_AREA_6_OFFSET</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E45" s="25"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="4" t="s">
+      <c r="E45" s="36"/>
+      <c r="F45" s="33"/>
+      <c r="G45" s="2" t="s">
         <v>128</v>
       </c>
       <c r="H45" s="2" t="str">
-        <f>A34</f>
+        <f t="shared" si="0"/>
         <v>RE_AREA_6_SIZE</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E46" s="25"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="4" t="s">
+      <c r="E46" s="36"/>
+      <c r="F46" s="33"/>
+      <c r="G46" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="H46" s="42" t="str">
+      <c r="H46" s="29" t="str">
         <f>A13</f>
         <v>RE_IMAGE_FLASH_APP_IMAGE_SIZE</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E47" s="25"/>
-      <c r="F47" s="48"/>
-      <c r="G47" s="4" t="s">
+      <c r="E47" s="36"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="H47" s="47" t="str">
+      <c r="H47" s="31" t="str">
         <f>A17</f>
         <v>RE_IMAGE_FLASH_DATA_IMAGE_SIZE</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E48" s="25"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="4" t="s">
+      <c r="E48" s="36"/>
+      <c r="F48" s="33"/>
+      <c r="G48" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H48" s="41" t="str">
+      <c r="H48" s="28" t="str">
         <f>A6</f>
         <v>RE_LOADER_CODE_START</v>
       </c>
     </row>
     <row r="49" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E49" s="26"/>
-      <c r="F49" s="23"/>
-      <c r="G49" s="4" t="s">
+      <c r="E49" s="37"/>
+      <c r="F49" s="34"/>
+      <c r="G49" s="2" t="s">
         <v>133</v>
       </c>
       <c r="H49" s="2" t="str">
@@ -3182,14 +3356,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="F35:F49"/>
-    <mergeCell ref="E19:E49"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F21:F24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="F27:F30"/>
-    <mergeCell ref="F33:F34"/>
     <mergeCell ref="G14:G15"/>
     <mergeCell ref="G16:G17"/>
     <mergeCell ref="F11:F18"/>
@@ -3199,7 +3365,1055 @@
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="F8:F10"/>
     <mergeCell ref="G12:G13"/>
+    <mergeCell ref="F35:F49"/>
+    <mergeCell ref="E19:E49"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F21:F24"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="F27:F30"/>
+    <mergeCell ref="F33:F34"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C038A9E-CEFD-4214-9C95-3A58D0A50079}">
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:N34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17.140625" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" customWidth="1"/>
+    <col min="13" max="13" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="43" t="s">
+        <v>160</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>175</v>
+      </c>
+      <c r="C9" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="43" t="s">
+        <v>161</v>
+      </c>
+      <c r="F9" s="43" t="s">
+        <v>162</v>
+      </c>
+      <c r="G9" s="43" t="s">
+        <v>174</v>
+      </c>
+      <c r="H9" s="43" t="s">
+        <v>164</v>
+      </c>
+      <c r="I9" s="43" t="s">
+        <v>163</v>
+      </c>
+      <c r="J9" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="K9" s="43" t="s">
+        <v>166</v>
+      </c>
+      <c r="L9" s="43" t="s">
+        <v>167</v>
+      </c>
+      <c r="M9" s="43" t="s">
+        <v>183</v>
+      </c>
+      <c r="N9" s="43" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="45">
+        <v>1</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" s="14">
+        <v>1</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J10" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M10" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N10" s="14" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="45">
+        <v>2</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J11" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K11" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M11" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N11" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="45">
+        <v>3</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F12" s="14">
+        <v>1</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J12" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K12" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M12" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N12" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="45">
+        <v>4</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F13" s="14">
+        <v>0</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J13" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K13" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M13" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N13" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="45">
+        <v>5</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F14" s="14">
+        <v>1</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J14" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K14" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M14" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N14" s="14" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="45">
+        <v>6</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F15" s="14">
+        <v>0</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J15" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K15" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M15" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N15" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="45">
+        <v>7</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F16" s="14">
+        <v>1</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L16" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M16" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N16" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="45">
+        <v>8</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F17" s="14">
+        <v>0</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L17" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M17" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N17" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="45">
+        <v>9</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F18" s="14">
+        <v>1</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J18" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K18" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L18" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M18" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N18" s="14" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="45">
+        <v>10</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F19" s="14">
+        <v>0</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J19" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K19" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L19" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M19" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N19" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="45">
+        <v>11</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F20" s="14">
+        <v>1</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H20" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I20" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J20" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K20" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L20" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M20" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N20" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="45">
+        <v>12</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F21" s="14">
+        <v>0</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J21" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K21" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L21" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M21" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N21" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="45">
+        <v>13</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F22" s="14">
+        <v>1</v>
+      </c>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N22" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="45">
+        <v>14</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F23" s="14">
+        <v>0</v>
+      </c>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M23" s="14"/>
+      <c r="N23" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="45">
+        <v>15</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F24" s="14">
+        <v>1</v>
+      </c>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="14"/>
+      <c r="M24" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N24" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="45">
+        <v>16</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F25" s="14">
+        <v>0</v>
+      </c>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M25" s="14"/>
+      <c r="N25" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="45">
+        <v>17</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F26" s="14">
+        <v>1</v>
+      </c>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="14"/>
+      <c r="K26" s="14"/>
+      <c r="L26" s="14"/>
+      <c r="M26" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N26" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="45">
+        <v>18</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F27" s="14">
+        <v>0</v>
+      </c>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14"/>
+      <c r="L27" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M27" s="14"/>
+      <c r="N27" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="45">
+        <v>19</v>
+      </c>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
+      <c r="M28" s="14"/>
+      <c r="N28" s="14"/>
+    </row>
+    <row r="29" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="45">
+        <v>20</v>
+      </c>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="14"/>
+      <c r="J29" s="14"/>
+      <c r="K29" s="14"/>
+      <c r="L29" s="14"/>
+      <c r="M29" s="14"/>
+      <c r="N29" s="14"/>
+    </row>
+    <row r="30" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="45">
+        <v>21</v>
+      </c>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14"/>
+      <c r="L30" s="14"/>
+      <c r="M30" s="14"/>
+      <c r="N30" s="14"/>
+    </row>
+    <row r="31" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="45">
+        <v>22</v>
+      </c>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
+      <c r="M31" s="14"/>
+      <c r="N31" s="14"/>
+    </row>
+    <row r="32" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="45">
+        <v>23</v>
+      </c>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="14"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14"/>
+      <c r="L32" s="14"/>
+      <c r="M32" s="14"/>
+      <c r="N32" s="14"/>
+    </row>
+    <row r="33" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="45">
+        <v>24</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="14"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
+      <c r="L33" s="14"/>
+      <c r="M33" s="14"/>
+      <c r="N33" s="14"/>
+    </row>
+    <row r="34" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="45">
+        <v>25</v>
+      </c>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
+      <c r="L34" s="14"/>
+      <c r="M34" s="14"/>
+      <c r="N34" s="14"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A9:L34" xr:uid="{0C038A9E-CEFD-4214-9C95-3A58D0A50079}">
+    <filterColumn colId="5">
+      <filters blank="1">
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <conditionalFormatting sqref="G10:N34">
+    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
+      <formula>$C$4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
+      <formula>$C$3</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
+      <formula>$C$1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
+      <formula>$C$2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10:E34">
+    <cfRule type="cellIs" dxfId="6" priority="6" operator="equal">
+      <formula>$A$2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
+      <formula>$A$1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F10:F34">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
+      <formula>$D$2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
+      <formula>$D$1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10:B34">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>$B$3</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>$B$2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>$B$1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10:E34" xr:uid="{1C05F047-0FFB-4DC0-9304-C7C5FAC3BCB7}">
+      <formula1>$A$1:$A$2</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F34" xr:uid="{CDCD4EAA-9FC2-48CE-99A6-116FE4353462}">
+      <formula1>$D$1:$D$2</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G10:N34" xr:uid="{E20357E7-74E1-4609-BC8C-8E9B4CD30CFC}">
+      <formula1>$C$1:$C$4</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10:B34" xr:uid="{DC7C77C6-B065-4670-B26D-05BC3F78FAEB}">
+      <formula1>$B$1:$B$3</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
OEMiROT (NTZ): Update OEMiROT_NTZ_flash_layout.xlsx with test result
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H563ZI/Applications/ROT_NTZ/OEMiROT_NTZ_flash_layout.xlsx
+++ b/Projects/NUCLEO-H563ZI/Applications/ROT_NTZ/OEMiROT_NTZ_flash_layout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ST\Cube\Cube1\STM32CubeH5\Projects\NUCLEO-H563ZI\Applications\ROT_NTZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E91070-8A6E-4E7C-B3A5-0E389C2D8964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D61B6FC-AEDF-4EC1-BA32-A70EE41712D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{973ADE99-8809-4282-875C-44A8EA15E93C}"/>
+    <workbookView xWindow="2685" yWindow="0" windowWidth="24360" windowHeight="15585" activeTab="2" xr2:uid="{973ADE99-8809-4282-875C-44A8EA15E93C}"/>
   </bookViews>
   <sheets>
     <sheet name="OEMiROT Flash Layout" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Test cases" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test cases'!$A$9:$L$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test cases'!$A$9:$L$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="185">
   <si>
     <t>offset</t>
   </si>
@@ -981,14 +981,27 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -999,89 +1012,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="17">
-    <dxf>
-      <font>
-        <color theme="6"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF0070C0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="6"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="6"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B0F0"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1116,6 +1060,62 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF00B0F0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="6"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0070C0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2528,10 +2528,10 @@
       <c r="B3" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="E3" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="F3" s="40" t="s">
+      <c r="F3" s="37" t="s">
         <v>87</v>
       </c>
       <c r="G3" s="16" t="s">
@@ -2552,8 +2552,8 @@
       <c r="C4" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="36"/>
-      <c r="F4" s="42"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="39"/>
       <c r="G4" s="16" t="s">
         <v>34</v>
       </c>
@@ -2572,8 +2572,8 @@
       <c r="C5" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="36"/>
-      <c r="F5" s="40" t="s">
+      <c r="E5" s="41"/>
+      <c r="F5" s="37" t="s">
         <v>88</v>
       </c>
       <c r="G5" s="16" t="s">
@@ -2594,8 +2594,8 @@
       <c r="C6" t="s">
         <v>55</v>
       </c>
-      <c r="E6" s="36"/>
-      <c r="F6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="38"/>
       <c r="G6" s="16" t="s">
         <v>89</v>
       </c>
@@ -2614,8 +2614,8 @@
       <c r="C7" t="s">
         <v>52</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="39"/>
       <c r="G7" s="2" t="s">
         <v>91</v>
       </c>
@@ -2634,10 +2634,10 @@
       <c r="C8" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="35" t="s">
+      <c r="E8" s="40" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="37" t="s">
         <v>59</v>
       </c>
       <c r="G8" s="16" t="s">
@@ -2658,8 +2658,8 @@
       <c r="C9" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="36"/>
-      <c r="F9" s="41"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="38"/>
       <c r="G9" s="16" t="s">
         <v>77</v>
       </c>
@@ -2678,8 +2678,8 @@
       <c r="C10" t="s">
         <v>147</v>
       </c>
-      <c r="E10" s="36"/>
-      <c r="F10" s="42"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="39"/>
       <c r="G10" s="16" t="s">
         <v>78</v>
       </c>
@@ -2698,8 +2698,8 @@
       <c r="C11" t="s">
         <v>145</v>
       </c>
-      <c r="E11" s="36"/>
-      <c r="F11" s="40" t="s">
+      <c r="E11" s="41"/>
+      <c r="F11" s="37" t="s">
         <v>56</v>
       </c>
       <c r="G11" s="16" t="s">
@@ -2720,9 +2720,9 @@
       <c r="C12" t="s">
         <v>146</v>
       </c>
-      <c r="E12" s="36"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="32" t="s">
+      <c r="E12" s="41"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="35" t="s">
         <v>64</v>
       </c>
       <c r="H12" s="25" t="str">
@@ -2740,9 +2740,9 @@
       <c r="C13" t="s">
         <v>148</v>
       </c>
-      <c r="E13" s="36"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="34"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="36"/>
       <c r="H13" s="25" t="str">
         <f>A20</f>
         <v>RE_BL2_WRP_END</v>
@@ -2758,9 +2758,9 @@
       <c r="C14" t="s">
         <v>149</v>
       </c>
-      <c r="E14" s="36"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="32" t="s">
+      <c r="E14" s="41"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="35" t="s">
         <v>83</v>
       </c>
       <c r="H14" s="21" t="str">
@@ -2778,9 +2778,9 @@
       <c r="C15" t="s">
         <v>149</v>
       </c>
-      <c r="E15" s="36"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="34"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="36"/>
       <c r="H15" s="21" t="str">
         <f>A9</f>
         <v>RE_LOADER_WRP_END</v>
@@ -2796,9 +2796,9 @@
       <c r="C16" t="s">
         <v>150</v>
       </c>
-      <c r="E16" s="36"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="32" t="s">
+      <c r="E16" s="41"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="35" t="s">
         <v>86</v>
       </c>
       <c r="H16" s="25" t="str">
@@ -2816,9 +2816,9 @@
       <c r="C17" t="s">
         <v>151</v>
       </c>
-      <c r="E17" s="36"/>
-      <c r="F17" s="41"/>
-      <c r="G17" s="34"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="36"/>
       <c r="H17" s="26" t="str">
         <f>A22</f>
         <v>RE_BL2_HDP_END</v>
@@ -2834,8 +2834,8 @@
       <c r="C18" t="s">
         <v>142</v>
       </c>
-      <c r="E18" s="37"/>
-      <c r="F18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="39"/>
       <c r="G18" s="27" t="s">
         <v>58</v>
       </c>
@@ -2854,10 +2854,10 @@
       <c r="C19" t="s">
         <v>143</v>
       </c>
-      <c r="E19" s="35" t="s">
+      <c r="E19" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="F19" s="32" t="s">
+      <c r="F19" s="35" t="s">
         <v>87</v>
       </c>
       <c r="G19" s="2" t="s">
@@ -2878,8 +2878,8 @@
       <c r="C20" t="s">
         <v>143</v>
       </c>
-      <c r="E20" s="36"/>
-      <c r="F20" s="34"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="36"/>
       <c r="G20" s="2" t="s">
         <v>91</v>
       </c>
@@ -2898,8 +2898,8 @@
       <c r="C21" t="s">
         <v>144</v>
       </c>
-      <c r="E21" s="36"/>
-      <c r="F21" s="32" t="s">
+      <c r="E21" s="41"/>
+      <c r="F21" s="35" t="s">
         <v>108</v>
       </c>
       <c r="G21" s="2" t="s">
@@ -2920,8 +2920,8 @@
       <c r="C22" t="s">
         <v>144</v>
       </c>
-      <c r="E22" s="36"/>
-      <c r="F22" s="33"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="43"/>
       <c r="G22" s="2" t="s">
         <v>99</v>
       </c>
@@ -2940,8 +2940,8 @@
       <c r="C23" t="s">
         <v>152</v>
       </c>
-      <c r="E23" s="36"/>
-      <c r="F23" s="33"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="43"/>
       <c r="G23" s="2" t="s">
         <v>100</v>
       </c>
@@ -2960,8 +2960,8 @@
       <c r="C24" t="s">
         <v>153</v>
       </c>
-      <c r="E24" s="36"/>
-      <c r="F24" s="34"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="36"/>
       <c r="G24" s="2" t="s">
         <v>101</v>
       </c>
@@ -2980,8 +2980,8 @@
       <c r="C25" t="s">
         <v>155</v>
       </c>
-      <c r="E25" s="36"/>
-      <c r="F25" s="32" t="s">
+      <c r="E25" s="41"/>
+      <c r="F25" s="35" t="s">
         <v>107</v>
       </c>
       <c r="G25" s="2" t="s">
@@ -3002,8 +3002,8 @@
       <c r="C26" t="s">
         <v>156</v>
       </c>
-      <c r="E26" s="36"/>
-      <c r="F26" s="34"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="36"/>
       <c r="G26" s="2" t="s">
         <v>95</v>
       </c>
@@ -3022,8 +3022,8 @@
       <c r="C27" t="s">
         <v>149</v>
       </c>
-      <c r="E27" s="36"/>
-      <c r="F27" s="32" t="s">
+      <c r="E27" s="41"/>
+      <c r="F27" s="35" t="s">
         <v>109</v>
       </c>
       <c r="G27" s="2" t="s">
@@ -3044,8 +3044,8 @@
       <c r="C28" t="s">
         <v>148</v>
       </c>
-      <c r="E28" s="36"/>
-      <c r="F28" s="33"/>
+      <c r="E28" s="41"/>
+      <c r="F28" s="43"/>
       <c r="G28" s="2" t="s">
         <v>99</v>
       </c>
@@ -3064,8 +3064,8 @@
       <c r="C29" t="s">
         <v>157</v>
       </c>
-      <c r="E29" s="36"/>
-      <c r="F29" s="33"/>
+      <c r="E29" s="41"/>
+      <c r="F29" s="43"/>
       <c r="G29" s="2" t="s">
         <v>100</v>
       </c>
@@ -3084,8 +3084,8 @@
       <c r="C30" t="s">
         <v>148</v>
       </c>
-      <c r="E30" s="36"/>
-      <c r="F30" s="34"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="36"/>
       <c r="G30" s="2" t="s">
         <v>101</v>
       </c>
@@ -3104,8 +3104,8 @@
       <c r="C31" t="s">
         <v>150</v>
       </c>
-      <c r="E31" s="36"/>
-      <c r="F31" s="32" t="s">
+      <c r="E31" s="41"/>
+      <c r="F31" s="35" t="s">
         <v>110</v>
       </c>
       <c r="G31" s="2" t="s">
@@ -3126,8 +3126,8 @@
       <c r="C32" t="s">
         <v>151</v>
       </c>
-      <c r="E32" s="36"/>
-      <c r="F32" s="34"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="36"/>
       <c r="G32" s="2" t="s">
         <v>95</v>
       </c>
@@ -3146,8 +3146,8 @@
       <c r="C33" t="s">
         <v>158</v>
       </c>
-      <c r="E33" s="36"/>
-      <c r="F33" s="38" t="s">
+      <c r="E33" s="41"/>
+      <c r="F33" s="44" t="s">
         <v>88</v>
       </c>
       <c r="G33" s="2" t="s">
@@ -3168,8 +3168,8 @@
       <c r="C34" t="s">
         <v>151</v>
       </c>
-      <c r="E34" s="36"/>
-      <c r="F34" s="39"/>
+      <c r="E34" s="41"/>
+      <c r="F34" s="45"/>
       <c r="G34" s="2" t="s">
         <v>91</v>
       </c>
@@ -3188,8 +3188,8 @@
       <c r="C35" t="s">
         <v>159</v>
       </c>
-      <c r="E35" s="36"/>
-      <c r="F35" s="32" t="s">
+      <c r="E35" s="41"/>
+      <c r="F35" s="35" t="s">
         <v>111</v>
       </c>
       <c r="G35" s="2" t="s">
@@ -3201,8 +3201,8 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E36" s="36"/>
-      <c r="F36" s="33"/>
+      <c r="E36" s="41"/>
+      <c r="F36" s="43"/>
       <c r="G36" s="2" t="s">
         <v>113</v>
       </c>
@@ -3212,8 +3212,8 @@
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E37" s="36"/>
-      <c r="F37" s="33"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="43"/>
       <c r="G37" s="2" t="s">
         <v>114</v>
       </c>
@@ -3223,8 +3223,8 @@
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E38" s="36"/>
-      <c r="F38" s="33"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="43"/>
       <c r="G38" s="2" t="s">
         <v>116</v>
       </c>
@@ -3234,8 +3234,8 @@
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E39" s="36"/>
-      <c r="F39" s="33"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="43"/>
       <c r="G39" s="2" t="s">
         <v>117</v>
       </c>
@@ -3245,8 +3245,8 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E40" s="36"/>
-      <c r="F40" s="33"/>
+      <c r="E40" s="41"/>
+      <c r="F40" s="43"/>
       <c r="G40" s="2" t="s">
         <v>119</v>
       </c>
@@ -3256,8 +3256,8 @@
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E41" s="36"/>
-      <c r="F41" s="33"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="43"/>
       <c r="G41" s="2" t="s">
         <v>120</v>
       </c>
@@ -3267,8 +3267,8 @@
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E42" s="36"/>
-      <c r="F42" s="33"/>
+      <c r="E42" s="41"/>
+      <c r="F42" s="43"/>
       <c r="G42" s="2" t="s">
         <v>123</v>
       </c>
@@ -3278,8 +3278,8 @@
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E43" s="36"/>
-      <c r="F43" s="33"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="43"/>
       <c r="G43" s="2" t="s">
         <v>124</v>
       </c>
@@ -3289,8 +3289,8 @@
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E44" s="36"/>
-      <c r="F44" s="33"/>
+      <c r="E44" s="41"/>
+      <c r="F44" s="43"/>
       <c r="G44" s="2" t="s">
         <v>127</v>
       </c>
@@ -3300,8 +3300,8 @@
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E45" s="36"/>
-      <c r="F45" s="33"/>
+      <c r="E45" s="41"/>
+      <c r="F45" s="43"/>
       <c r="G45" s="2" t="s">
         <v>128</v>
       </c>
@@ -3311,8 +3311,8 @@
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E46" s="36"/>
-      <c r="F46" s="33"/>
+      <c r="E46" s="41"/>
+      <c r="F46" s="43"/>
       <c r="G46" s="2" t="s">
         <v>131</v>
       </c>
@@ -3322,8 +3322,8 @@
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E47" s="36"/>
-      <c r="F47" s="33"/>
+      <c r="E47" s="41"/>
+      <c r="F47" s="43"/>
       <c r="G47" s="2" t="s">
         <v>132</v>
       </c>
@@ -3333,8 +3333,8 @@
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E48" s="36"/>
-      <c r="F48" s="33"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="43"/>
       <c r="G48" s="2" t="s">
         <v>49</v>
       </c>
@@ -3344,8 +3344,8 @@
       </c>
     </row>
     <row r="49" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E49" s="37"/>
-      <c r="F49" s="34"/>
+      <c r="E49" s="42"/>
+      <c r="F49" s="36"/>
       <c r="G49" s="2" t="s">
         <v>133</v>
       </c>
@@ -3356,6 +3356,14 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="F35:F49"/>
+    <mergeCell ref="E19:E49"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F21:F24"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="F27:F30"/>
+    <mergeCell ref="F33:F34"/>
     <mergeCell ref="G14:G15"/>
     <mergeCell ref="G16:G17"/>
     <mergeCell ref="F11:F18"/>
@@ -3365,14 +3373,6 @@
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="F8:F10"/>
     <mergeCell ref="G12:G13"/>
-    <mergeCell ref="F35:F49"/>
-    <mergeCell ref="E19:E49"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F21:F24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="F27:F30"/>
-    <mergeCell ref="F33:F34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3380,8 +3380,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C038A9E-CEFD-4214-9C95-3A58D0A50079}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -3400,7 +3399,7 @@
     <col min="14" max="14" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>168</v>
       </c>
@@ -3414,7 +3413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>169</v>
       </c>
@@ -3428,7 +3427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>178</v>
       </c>
@@ -3436,7 +3435,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>173</v>
       </c>
@@ -3462,51 +3461,51 @@
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="32" t="s">
         <v>160</v>
       </c>
-      <c r="B9" s="44" t="s">
+      <c r="B9" s="33" t="s">
         <v>175</v>
       </c>
-      <c r="C9" s="43" t="s">
+      <c r="C9" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="43" t="s">
+      <c r="E9" s="32" t="s">
         <v>161</v>
       </c>
-      <c r="F9" s="43" t="s">
+      <c r="F9" s="32" t="s">
         <v>162</v>
       </c>
-      <c r="G9" s="43" t="s">
+      <c r="G9" s="32" t="s">
         <v>174</v>
       </c>
-      <c r="H9" s="43" t="s">
+      <c r="H9" s="32" t="s">
         <v>164</v>
       </c>
-      <c r="I9" s="43" t="s">
+      <c r="I9" s="32" t="s">
         <v>163</v>
       </c>
-      <c r="J9" s="43" t="s">
+      <c r="J9" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="K9" s="43" t="s">
+      <c r="K9" s="32" t="s">
         <v>166</v>
       </c>
-      <c r="L9" s="43" t="s">
+      <c r="L9" s="32" t="s">
         <v>167</v>
       </c>
-      <c r="M9" s="43" t="s">
+      <c r="M9" s="32" t="s">
         <v>183</v>
       </c>
-      <c r="N9" s="43" t="s">
+      <c r="N9" s="32" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="45">
+      <c r="A10" s="34">
         <v>1</v>
       </c>
       <c r="B10" s="14" t="s">
@@ -3549,8 +3548,8 @@
         <v>170</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="45">
+    <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="34">
         <v>2</v>
       </c>
       <c r="B11" s="14" t="s">
@@ -3594,7 +3593,7 @@
       </c>
     </row>
     <row r="12" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="45">
+      <c r="A12" s="34">
         <v>3</v>
       </c>
       <c r="B12" s="14" t="s">
@@ -3637,8 +3636,8 @@
         <v>172</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="45">
+    <row r="13" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="34">
         <v>4</v>
       </c>
       <c r="B13" s="14" t="s">
@@ -3682,7 +3681,7 @@
       </c>
     </row>
     <row r="14" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="45">
+      <c r="A14" s="34">
         <v>5</v>
       </c>
       <c r="B14" s="14" t="s">
@@ -3725,8 +3724,8 @@
         <v>170</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="45">
+    <row r="15" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="34">
         <v>6</v>
       </c>
       <c r="B15" s="14" t="s">
@@ -3770,7 +3769,7 @@
       </c>
     </row>
     <row r="16" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="45">
+      <c r="A16" s="34">
         <v>7</v>
       </c>
       <c r="B16" s="14" t="s">
@@ -3813,8 +3812,8 @@
         <v>172</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="45">
+    <row r="17" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="34">
         <v>8</v>
       </c>
       <c r="B17" s="14" t="s">
@@ -3858,7 +3857,7 @@
       </c>
     </row>
     <row r="18" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="45">
+      <c r="A18" s="34">
         <v>9</v>
       </c>
       <c r="B18" s="14" t="s">
@@ -3901,8 +3900,8 @@
         <v>170</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="45">
+    <row r="19" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="34">
         <v>10</v>
       </c>
       <c r="B19" s="14" t="s">
@@ -3946,7 +3945,7 @@
       </c>
     </row>
     <row r="20" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="45">
+      <c r="A20" s="34">
         <v>11</v>
       </c>
       <c r="B20" s="14" t="s">
@@ -3989,8 +3988,8 @@
         <v>172</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="45">
+    <row r="21" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="34">
         <v>12</v>
       </c>
       <c r="B21" s="14" t="s">
@@ -4034,7 +4033,7 @@
       </c>
     </row>
     <row r="22" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="45">
+      <c r="A22" s="34">
         <v>13</v>
       </c>
       <c r="B22" s="14" t="s">
@@ -4052,12 +4051,24 @@
       <c r="F22" s="14">
         <v>1</v>
       </c>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
+      <c r="G22" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H22" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I22" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J22" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K22" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L22" s="14" t="s">
+        <v>170</v>
+      </c>
       <c r="M22" s="14" t="s">
         <v>172</v>
       </c>
@@ -4065,8 +4076,8 @@
         <v>172</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="45">
+    <row r="23" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="34">
         <v>14</v>
       </c>
       <c r="B23" s="14" t="s">
@@ -4084,21 +4095,33 @@
       <c r="F23" s="14">
         <v>0</v>
       </c>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="14"/>
+      <c r="G23" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H23" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J23" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K23" s="14" t="s">
+        <v>170</v>
+      </c>
       <c r="L23" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="M23" s="14"/>
+      <c r="M23" s="14" t="s">
+        <v>172</v>
+      </c>
       <c r="N23" s="14" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="45">
+      <c r="A24" s="34">
         <v>15</v>
       </c>
       <c r="B24" s="14" t="s">
@@ -4116,12 +4139,24 @@
       <c r="F24" s="14">
         <v>1</v>
       </c>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
+      <c r="G24" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J24" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K24" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L24" s="14" t="s">
+        <v>170</v>
+      </c>
       <c r="M24" s="14" t="s">
         <v>172</v>
       </c>
@@ -4129,8 +4164,8 @@
         <v>172</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="45">
+    <row r="25" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="34">
         <v>16</v>
       </c>
       <c r="B25" s="14" t="s">
@@ -4148,21 +4183,33 @@
       <c r="F25" s="14">
         <v>0</v>
       </c>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
+      <c r="G25" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J25" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K25" s="14" t="s">
+        <v>170</v>
+      </c>
       <c r="L25" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="M25" s="14"/>
+      <c r="M25" s="14" t="s">
+        <v>172</v>
+      </c>
       <c r="N25" s="14" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="45">
+      <c r="A26" s="34">
         <v>17</v>
       </c>
       <c r="B26" s="14" t="s">
@@ -4180,12 +4227,24 @@
       <c r="F26" s="14">
         <v>1</v>
       </c>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
-      <c r="L26" s="14"/>
+      <c r="G26" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J26" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K26" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L26" s="14" t="s">
+        <v>170</v>
+      </c>
       <c r="M26" s="14" t="s">
         <v>172</v>
       </c>
@@ -4193,8 +4252,8 @@
         <v>172</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="45">
+    <row r="27" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="34">
         <v>18</v>
       </c>
       <c r="B27" s="14" t="s">
@@ -4212,205 +4271,893 @@
       <c r="F27" s="14">
         <v>0</v>
       </c>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
+      <c r="G27" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I27" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J27" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K27" s="14" t="s">
+        <v>170</v>
+      </c>
       <c r="L27" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="M27" s="14"/>
+      <c r="M27" s="14" t="s">
+        <v>172</v>
+      </c>
       <c r="N27" s="14" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="45">
+      <c r="A28" s="34">
         <v>19</v>
       </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14"/>
-      <c r="K28" s="14"/>
-      <c r="L28" s="14"/>
-      <c r="M28" s="14"/>
-      <c r="N28" s="14"/>
+      <c r="B28" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F28" s="14">
+        <v>1</v>
+      </c>
+      <c r="G28" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H28" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I28" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J28" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K28" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L28" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M28" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N28" s="14" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="29" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="45">
+      <c r="A29" s="34">
         <v>20</v>
       </c>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="14"/>
-      <c r="M29" s="14"/>
-      <c r="N29" s="14"/>
+      <c r="B29" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F29" s="14">
+        <v>0</v>
+      </c>
+      <c r="G29" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H29" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J29" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K29" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L29" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M29" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N29" s="14" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="30" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="45">
+      <c r="A30" s="34">
         <v>21</v>
       </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="14"/>
-      <c r="K30" s="14"/>
-      <c r="L30" s="14"/>
-      <c r="M30" s="14"/>
-      <c r="N30" s="14"/>
+      <c r="B30" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F30" s="14">
+        <v>1</v>
+      </c>
+      <c r="G30" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H30" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J30" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K30" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L30" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M30" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N30" s="14" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="31" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="45">
+      <c r="A31" s="34">
         <v>22</v>
       </c>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
-      <c r="M31" s="14"/>
-      <c r="N31" s="14"/>
+      <c r="B31" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F31" s="14">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H31" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I31" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J31" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K31" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L31" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M31" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N31" s="14" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="32" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="45">
+      <c r="A32" s="34">
         <v>23</v>
       </c>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="14"/>
-      <c r="K32" s="14"/>
-      <c r="L32" s="14"/>
-      <c r="M32" s="14"/>
-      <c r="N32" s="14"/>
+      <c r="B32" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F32" s="14">
+        <v>1</v>
+      </c>
+      <c r="G32" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J32" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K32" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L32" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M32" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N32" s="14" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="33" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="45">
+      <c r="A33" s="34">
         <v>24</v>
       </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="14"/>
-      <c r="M33" s="14"/>
-      <c r="N33" s="14"/>
+      <c r="B33" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F33" s="14">
+        <v>0</v>
+      </c>
+      <c r="G33" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H33" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I33" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J33" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K33" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L33" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M33" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="N33" s="14" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="34" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="45">
+      <c r="A34" s="34">
         <v>25</v>
       </c>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="14"/>
-      <c r="J34" s="14"/>
-      <c r="K34" s="14"/>
-      <c r="L34" s="14"/>
-      <c r="M34" s="14"/>
-      <c r="N34" s="14"/>
+      <c r="B34" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F34" s="14">
+        <v>1</v>
+      </c>
+      <c r="G34" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I34" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J34" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K34" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L34" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M34" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N34" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="34">
+        <v>26</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F35" s="14">
+        <v>0</v>
+      </c>
+      <c r="G35" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H35" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I35" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J35" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K35" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L35" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M35" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N35" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="34">
+        <v>27</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F36" s="14">
+        <v>1</v>
+      </c>
+      <c r="G36" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H36" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J36" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K36" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L36" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M36" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N36" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="34">
+        <v>28</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F37" s="14">
+        <v>0</v>
+      </c>
+      <c r="G37" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H37" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I37" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J37" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K37" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L37" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M37" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N37" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="34">
+        <v>29</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F38" s="14">
+        <v>1</v>
+      </c>
+      <c r="G38" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J38" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K38" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L38" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M38" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N38" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="34">
+        <v>30</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E39" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F39" s="14">
+        <v>0</v>
+      </c>
+      <c r="G39" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H39" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I39" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J39" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K39" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L39" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M39" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N39" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="34">
+        <v>31</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E40" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F40" s="14">
+        <v>0</v>
+      </c>
+      <c r="G40" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H40" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I40" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J40" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K40" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L40" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M40" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N40" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="34">
+        <v>32</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C41" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F41" s="14">
+        <v>1</v>
+      </c>
+      <c r="G41" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H41" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I41" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J41" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K41" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L41" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M41" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N41" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="34">
+        <v>33</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E42" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F42" s="14">
+        <v>0</v>
+      </c>
+      <c r="G42" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H42" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I42" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J42" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K42" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L42" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M42" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N42" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A43" s="34">
+        <v>34</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E43" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F43" s="14">
+        <v>1</v>
+      </c>
+      <c r="G43" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H43" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I43" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J43" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K43" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L43" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M43" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N43" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A44" s="34">
+        <v>35</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C44" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F44" s="14">
+        <v>0</v>
+      </c>
+      <c r="G44" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H44" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I44" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J44" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K44" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L44" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="M44" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N44" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A45" s="34">
+        <v>36</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E45" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F45" s="14">
+        <v>1</v>
+      </c>
+      <c r="G45" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="H45" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="I45" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="J45" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="K45" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="L45" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="M45" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="N45" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A46" s="34"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="14"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="14"/>
+      <c r="J46" s="14"/>
+      <c r="K46" s="14"/>
+      <c r="L46" s="14"/>
+      <c r="M46" s="14"/>
+      <c r="N46" s="14"/>
     </row>
   </sheetData>
-  <autoFilter ref="A9:L34" xr:uid="{0C038A9E-CEFD-4214-9C95-3A58D0A50079}">
-    <filterColumn colId="5">
-      <filters blank="1">
-        <filter val="1"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <conditionalFormatting sqref="G10:N34">
-    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
+  <autoFilter ref="A9:L46" xr:uid="{0C038A9E-CEFD-4214-9C95-3A58D0A50079}"/>
+  <conditionalFormatting sqref="B10:B46">
+    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
+      <formula>$B$3</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
+      <formula>$B$2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="3" operator="equal">
+      <formula>$B$1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10:E46">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="equal">
+      <formula>$A$2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+      <formula>$A$1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F10:F46">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>$D$2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>$D$1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G10:N46">
+    <cfRule type="cellIs" dxfId="3" priority="8" operator="equal">
       <formula>$C$4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="9" operator="equal">
       <formula>$C$3</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="10" operator="equal">
       <formula>$C$1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="11" operator="equal">
       <formula>$C$2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C10:E34">
-    <cfRule type="cellIs" dxfId="6" priority="6" operator="equal">
-      <formula>$A$2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
-      <formula>$A$1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F10:F34">
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
-      <formula>$D$2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
-      <formula>$D$1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B10:B34">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
-      <formula>$B$3</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>$B$2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
-      <formula>$B$1</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10:E34" xr:uid="{1C05F047-0FFB-4DC0-9304-C7C5FAC3BCB7}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10:E46" xr:uid="{1C05F047-0FFB-4DC0-9304-C7C5FAC3BCB7}">
       <formula1>$A$1:$A$2</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F34" xr:uid="{CDCD4EAA-9FC2-48CE-99A6-116FE4353462}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F46" xr:uid="{CDCD4EAA-9FC2-48CE-99A6-116FE4353462}">
       <formula1>$D$1:$D$2</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G10:N34" xr:uid="{E20357E7-74E1-4609-BC8C-8E9B4CD30CFC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G10:N46" xr:uid="{E20357E7-74E1-4609-BC8C-8E9B4CD30CFC}">
       <formula1>$C$1:$C$4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10:B34" xr:uid="{DC7C77C6-B065-4670-B26D-05BC3F78FAEB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10:B46" xr:uid="{DC7C77C6-B065-4670-B26D-05BC3F78FAEB}">
       <formula1>$B$1:$B$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>